<commit_message>
Update knowledge base with 128 Q&As
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="الأسئلة والأجوبة" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B110"/>
+  <dimension ref="A1:B134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>الأسئلة والأجوبة الخاصة بكلية علوم الحاسوب</t>
+          <t>الأسئلة والأجوبة الخاصة بكلية علوم الحاسوب وتقانة المعلومات</t>
         </is>
       </c>
     </row>
@@ -438,1296 +442,1584 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>كيف أدخل إلى نظام التسجيل؟</t>
+          <t>كيف أسجل؟</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>دخول عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>هل التسجيل إلكتروني أم حضوري؟</t>
+          <t>كيف أسجل في الكلية؟</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>التسجيل إلكتروني عبر الموقع الرسمي للجامعة</t>
+          <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>كيف أكمل إجراءات التسجيل؟</t>
+          <t>كيف أسجل في الجامعة؟</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ملء 4 خطوات: المعلومات الأساسية، أولياء الأمور، القبول، الأكاديمية، ثم التحقق من الهاتف والبريد الإلكتروني</t>
+          <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>كيف أتأكد أن تسجيلي اكتمل؟</t>
+          <t>كيف أتسجل؟</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>يصل رمز تحقق من 4 أرقام على الهاتف، ورسالة على البريد الإلكتروني</t>
+          <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ما البيانات المطلوبة في استمارة التسجيل؟</t>
+          <t>كيف اسجل؟</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>الاسم بالعربي والإنجليزي، صورة شخصية، رقم الهاتف، البريد الإلكتروني، عنوان المنزل، الرقم الوطني، المدينة، المنطقة</t>
+          <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ما الخطوة الأولى في التسجيل؟</t>
+          <t>كيف اسجل في الكلية؟</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>كتابة الاسم الكامل بالعربي والإنجليزي، مع صورة شخصية، ورقم الهاتف، والبريد الإلكتروني، وعنوان المنزل</t>
+          <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ما الخطوة الثانية في التسجيل؟</t>
+          <t>كيف اسجل في الجامعة؟</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>إدخال معلومات أولياء الأمور</t>
+          <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ما الخطوة الثالثة في التسجيل؟</t>
+          <t>اريد اسجل</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>اختيار معايير الترشيح للقبول: عن طريق مكتب وزارة التعليم العالي، أو عن طريق الجامعة</t>
+          <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ما الخطوة الرابعة في التسجيل؟</t>
+          <t>عايز اسجل</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>إدخال المعلومات الأكاديمية: رقم الجلوس، اسم المدرسة، المسار المختار، إرفاق نسخة من شهادة الثانوية</t>
+          <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ما الذي يجب فعله بعد ملء الاستمارة؟</t>
+          <t>كيف أقدم؟</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>تجاوز reCaptcha (أنا لست روبوتاً)، ثم الضغط على إرسال</t>
+          <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ما الذي يحدث بعد إرسال الاستمارة؟</t>
+          <t>كيف أقدم على الجامعة؟</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>يُرسل رمز تحقق من 4 أرقام على الهاتف، ورسالة على البريد الإلكتروني</t>
+          <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ماذا يحدث بعد التسجيل؟</t>
+          <t>كيف أقدم في الكلية؟</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>يُنشئ النظام حساباً للطالب باستخدام البريد الإلكتروني المُقدَّم، ويُرسل رابطاً لإنشاء كلمة مرور جديدة</t>
+          <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>كيف يدخل الطالب بعد التسجيل؟</t>
+          <t>كيف اقدم؟</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
+          <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ماذا أفعل بعد اكتمال التسجيل؟</t>
+          <t>اريد اقدم</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>تُرسل رسالة من الجامعة على البريد الإلكتروني المُسجَّل به، فيها الخطوات التالية</t>
+          <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ما الخطوة التالية بعد التسجيل؟</t>
+          <t>عايز اقدم</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>تُرسل رسالة من الجامعة على البريد الإلكتروني بعد القبول، فيها الخطوات التالية</t>
+          <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ما شروط القبول العامة في الجامعة؟</t>
+          <t>اين اسجل؟</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>استيفاء شروط القبول العامة التي يقرها المجلس القومي للتعليم العالي والبحث العلمي</t>
+          <t>التسجيل إلكتروني عبر الموقع: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>هل توجد شروط إضافية للقبول؟</t>
+          <t>اين اقدم؟</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>استيفاء أي شروط أخرى تحددها الجامعة أو الكلية</t>
+          <t>التقديم إلكتروني عبر الموقع: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>هل هناك اختبار للقبول؟</t>
+          <t>ما هو موقع التسجيل؟</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>اجتياز اختبار أو معاينة شخصية وفق ما تحدده الكلية</t>
+          <t>https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ما الشروط الأساسية للقبول في كلية الحاسوب؟</t>
+          <t>ما رابط التسجيل؟</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>الحصول على الشهادة السودانية أو ما يعادلها، النجاح في المواد المؤهلة، اجتياز اختبارات القبول والمعاينة، موافقة الوزارة</t>
+          <t>https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ما المواد المطلوبة للقبول في كلية علوم الحاسوب؟</t>
+          <t>ما رابط التقديم؟</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>اللغة العربية، اللغة الإنجليزية، التربية الدينية، الرياضيات، الكيمياء، الفيزياء + أفضل مادة من (الأحياء، علوم الحاسوب، العلوم الهندسية)</t>
+          <t>https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ما هي أقسام كلية علوم الحاسوب وتقانة المعلومات؟</t>
+          <t>كيف أدخل إلى نظام التسجيل؟</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>علوم الحاسوب (تخصص الذكاء الاصطناعي وعلم البيانات)، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، الدبلوم في تقنية المعلومات</t>
+          <t>دخول عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ما هي البرامج المتاحة في كلية علوم الحاسوب؟</t>
+          <t>هل التسجيل إلكتروني أم حضوري؟</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>بكالوريوس الشرف في علوم الحاسوب، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، دبلوم في تقنية المعلومات</t>
+          <t>التسجيل إلكتروني عبر الموقع الرسمي للجامعة</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ما هو بكالوريوس الشرف في علوم الحاسوب - الذكاء الاصطناعي؟</t>
+          <t>كيف أكمل إجراءات التسجيل؟</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>برنامج لمدة 4 سنوات، يشمل التعلم الآلي، التعلم العميق، معالجة اللغات الطبيعية، الرؤية الحاسوبية، والروبوتات</t>
+          <t>ملء 4 خطوات: المعلومات الأساسية، أولياء الأمور، القبول، الأكاديمية، ثم التحقق من الهاتف والبريد الإلكتروني</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ما هو بكالوريوس الشرف في علوم الحاسوب - علم البيانات؟</t>
+          <t>كيف أتأكد أن تسجيلي اكتمل؟</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>برنامج لمدة 4 سنوات، يركز على دورة حياة البيانات بالكامل</t>
+          <t>يصل رمز تحقق من 4 أرقام على الهاتف، ورسالة على البريد الإلكتروني</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ما هو بكالوريوس الشرف في تكنولوجيا المعلومات والاتصالات؟</t>
+          <t>ما البيانات المطلوبة في استمارة التسجيل؟</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>برنامج لمدة 4 سنوات، يؤهل متخصصين في الشبكات، الأمن السيبراني، وإدارة الأنظمة</t>
+          <t>الاسم بالعربي والإنجليزي، صورة شخصية، رقم الهاتف، البريد الإلكتروني، عنوان المنزل، الرقم الوطني، المدينة، المنطقة</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ما هو بكالوريوس الشرف في تقنية المعلومات؟</t>
+          <t>ما الخطوة الأولى في التسجيل؟</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>برنامج لمدة 4 سنوات، يركز على إدارة الأنظمة، الشبكات، أمن المعلومات، وتطوير التطبيقات</t>
+          <t>كتابة الاسم الكامل بالعربي والإنجليزي، مع صورة شخصية، ورقم الهاتف، والبريد الإلكتروني، وعنوان المنزل</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ما هي فرص العمل لخريجي علوم الحاسوب؟</t>
+          <t>ما الخطوة الثانية في التسجيل؟</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>مطور تطبيقات ذكاء اصطناعي، مهندس تعلم آلي، عالم بيانات، مطور أنظمة ذكية، مهندس شبكات، مدير أنظمة، محلل أمن معلومات</t>
+          <t>إدخال معلومات أولياء الأمور</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ما مطلوبات التقديم لكلية الحاسوب؟</t>
+          <t>ما الخطوة الثالثة في التسجيل؟</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ملء طلب الالتحاق، النجاح في المواد المؤهلة، أصل وصورة من الشهادة السودانية، أصل وصورة من الرقم الوطني</t>
+          <t>اختيار معايير الترشيح للقبول: عن طريق مكتب وزارة التعليم العالي، أو عن طريق الجامعة</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ما المستندات المطلوبة للتسجيل؟</t>
+          <t>ما الخطوة الرابعة في التسجيل؟</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ملء طلب الالتحاق + أصل وصورة الشهادة السودانية + أصل وصورة الرقم الوطني + صورة شخصية</t>
+          <t>إدخال المعلومات الأكاديمية: رقم الجلوس، اسم المدرسة، المسار المختار، إرفاق نسخة من شهادة الثانوية</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>هل أحتاج صور شخصية؟</t>
+          <t>ما الذي يجب فعله بعد ملء الاستمارة؟</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>نعم، صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
+          <t>تجاوز reCaptcha (أنا لست روبوتاً)، ثم الضغط على إرسال</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>هل أحتاج إثبات هوية؟</t>
+          <t>ما الذي يحدث بعد إرسال الاستمارة؟</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>نعم، الرقم الوطني</t>
+          <t>يُرسل رمز تحقق من 4 أرقام على الهاتف، ورسالة على البريد الإلكتروني</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ما نوع إثبات الهوية المطلوب؟</t>
+          <t>ماذا يحدث بعد التسجيل؟</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>الرقم الوطني أو جواز السفر</t>
+          <t>يُنشئ النظام حساباً للطالب باستخدام البريد الإلكتروني المُقدَّم، ويُرسل رابطاً لإنشاء كلمة مرور جديدة</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>هل أحتاج شهادة الثانوية؟</t>
+          <t>كيف يدخل الطالب بعد التسجيل؟</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>نعم، أصل وصورة من الشهادة السودانية أو ما يعادلها</t>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>هل أحتاج امتحان قدرات؟</t>
+          <t>ماذا أفعل بعد اكتمال التسجيل؟</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>نعم، لشهادة السعودية (امتحان القدرات والتحصيل)</t>
+          <t>تُرسل رسالة من الجامعة على البريد الإلكتروني المُسجَّل به، فيها الخطوات التالية</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>أين يتم التقديم؟</t>
+          <t>ما الخطوة التالية بعد التسجيل؟</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>التقديم والتسجيل أون لاين عبر الموقع الإلكتروني</t>
+          <t>تُرسل رسالة من الجامعة على البريد الإلكتروني بعد القبول، فيها الخطوات التالية</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>أين مكتب القبول؟</t>
+          <t>ما شروط القبول العامة في الجامعة؟</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+          <t>استيفاء شروط القبول العامة التي يقرها المجلس القومي للتعليم العالي والبحث العلمي</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ما شروط التحويل من جامعة أخرى إلى كلية الحاسوب في UST؟</t>
+          <t>هل توجد شروط إضافية للقبول؟</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>التحويل من الكلية المحول منها إلى ما يناظرها في UST</t>
+          <t>استيفاء أي شروط أخرى تحددها الجامعة أو الكلية</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ما شرط النسبة المئوية للتحويل؟</t>
+          <t>هل هناك اختبار للقبول؟</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>لا تقل النسبة المئوية في الشهادة الثانوية عن النسبة المحددة للكلية المناظرة</t>
+          <t>اجتياز اختبار أو معاينة شخصية وفق ما تحدده الكلية</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ما شروط التحويل لكلية علوم الحاسوب؟</t>
+          <t>ما الشروط الأساسية للقبول في كلية الحاسوب؟</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>السنة الثالثة أو ما دونها</t>
+          <t>الحصول على الشهادة السودانية أو ما يعادلها، النجاح في المواد المؤهلة، اجتياز اختبارات القبول والمعاينة، موافقة الوزارة</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ما الوثائق المطلوبة للتحويل؟</t>
+          <t>ما المواد المطلوبة للقبول في كلية علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>الشهادة الثانوية، صورة جواز السفر أو الرقم الوطني، شهادة التفاصيل من الكلية المحول منها</t>
+          <t>اللغة العربية، اللغة الإنجليزية، التربية الدينية، الرياضيات، الكيمياء، الفيزياء + أفضل مادة من (الأحياء، علوم الحاسوب، العلوم الهندسية)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>كيف أحوّل إلى كلية أخرى داخل UST؟</t>
+          <t>ما هي أقسام كلية علوم الحاسوب وتقانة المعلومات؟</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>عبر الرابط: reg.ust.edu.sd/ust/online/transfer</t>
+          <t>علوم الحاسوب (تخصص الذكاء الاصطناعي وعلم البيانات)، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، الدبلوم في تقنية المعلومات</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>كيف أحوّل من جامعة أخرى إلى UST؟</t>
+          <t>ما هي أقسام كلية الحاسوب؟</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>عبر الرابط: reg.ust.edu.sd/student/submit/new_internal</t>
+          <t>علوم الحاسوب، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، الدبلوم في تقنية المعلومات</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ما رابط التحويل؟</t>
+          <t>ما هي تخصصات كلية الحاسوب؟</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>reg.ust.edu.sd/ust/online/transfer</t>
+          <t>علوم الحاسوب (ذكاء اصطناعي وعلم بيانات)، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ما شروط القبول للماجستير؟</t>
+          <t>ما هي البرامج المتاحة في كلية علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>الحصول على درجة البكالوريوس بمرتبة الشرف أو ما يعادلها في التخصص المعني من جامعة معترف بها</t>
+          <t>بكالوريوس الشرف في علوم الحاسوب، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، دبلوم في تقنية المعلومات</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ماذا لو لم يحصل الطالب على مرتبة الشرف؟</t>
+          <t>ما هو بكالوريوس الشرف في علوم الحاسوب - الذكاء الاصطناعي؟</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>يُشترط: دبلوم عالي مميز في مجال التخصص، أو خبرة مناسبة في المجال، أو قضاء عام دراسي تأهيلي</t>
+          <t>برنامج لمدة 4 سنوات، يشمل التعلم الآلي، التعلم العميق، معالجة اللغات الطبيعية، الرؤية الحاسوبية، والروبوتات</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>هل يمكن التسجيل بتفرغ جزئي أو كلي؟</t>
+          <t>ما هو بكالوريوس الشرف في علوم الحاسوب - علم البيانات؟</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>نعم، حسب شروط لوائح الدرجة المعنية</t>
+          <t>برنامج لمدة 4 سنوات، يركز على دورة حياة البيانات بالكامل</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ما شروط القبول للدكتوراة؟</t>
+          <t>ما هو بكالوريوس الشرف في تكنولوجيا المعلومات والاتصالات؟</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>الحصول على درجة الماجستير من جامعة معترف بها</t>
+          <t>برنامج لمدة 4 سنوات، يؤهل متخصصين في الشبكات، الأمن السيبراني، وإدارة الأنظمة</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>كم مدة دراسة الدكتوراة؟</t>
+          <t>ما هو بكالوريوس الشرف في تقنية المعلومات؟</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>لا تقل عن عامين (ثلاثة أعوام للتفرغ الجزئي)، ولا تزيد عن خمسة أعوام</t>
+          <t>برنامج لمدة 4 سنوات، يركز على إدارة الأنظمة، الشبكات، أمن المعلومات، وتطوير التطبيقات</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ما برامج الدراسات العليا في كلية علوم الحاسوب؟</t>
+          <t>ما هي فرص العمل لخريجي علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>الماجستير بالمقررات في علوم الحاسوب، تقنية المعلومات، نظم المعلومات، أمن المعلومات + دبلوم عالي في علوم الحاسوب</t>
+          <t>مطور تطبيقات ذكاء اصطناعي، مهندس تعلم آلي، عالم بيانات، مطور أنظمة ذكية، مهندس شبكات، مدير أنظمة، محلل أمن معلومات</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ما رابط التقديم للدراسات العليا؟</t>
+          <t>ما مطلوبات التقديم لكلية الحاسوب؟</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>reg.ust.edu.sd/student/submit/new_postgraduate</t>
+          <t>ملء طلب الالتحاق، النجاح في المواد المؤهلة، أصل وصورة من الشهادة السودانية، أصل وصورة من الرقم الوطني</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ما شروط القبول لماجستير أمن المعلومات؟</t>
+          <t>ما المستندات المطلوبة للتسجيل؟</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
+          <t>ملء طلب الالتحاق + أصل وصورة الشهادة السودانية + أصل وصورة الرقم الوطني + صورة شخصية</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ما شروط القبول لماجستير تقنية المعلومات؟</t>
+          <t>هل أحتاج صور شخصية؟</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
+          <t>نعم، صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ما شروط القبول لماجستير علوم الحاسوب؟</t>
+          <t>ما صيغة الصورة الشخصية المطلوبة؟</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
+          <t>صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (سوداني - السودان)؟</t>
+          <t>هل أحتاج إثبات هوية؟</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>نعم، الرقم الوطني</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (سوداني - مصر)؟</t>
+          <t>ما نوع إثبات الهوية المطلوب؟</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>الرقم الوطني أو جواز السفر</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (سوداني - السعودية)؟</t>
+          <t>هل أحتاج شهادة الثانوية؟</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>9,020 درهم (إجمالي الرسوم)</t>
+          <t>نعم، أصل وصورة من الشهادة السودانية أو ما يعادلها</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السودان)؟</t>
+          <t>هل أحتاج امتحان قدرات؟</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>نعم، لشهادة السعودية (امتحان القدرات والتحصيل)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - مصر)؟</t>
+          <t>أين يتم التقديم؟</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>التقديم والتسجيل أون لاين عبر الموقع الإلكتروني</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السعودية)؟</t>
+          <t>أين مكتب القبول؟</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>15,640 درهم (إجمالي الرسوم)</t>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السودان)؟</t>
+          <t>ما شروط التحويل من جامعة أخرى إلى كلية الحاسوب في UST؟</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>التحويل من الكلية المحول منها إلى ما يناظرها في UST</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - مصر)؟</t>
+          <t>ما شرط النسبة المئوية للتحويل؟</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>لا تقل النسبة المئوية في الشهادة الثانوية عن النسبة المحددة للكلية المناظرة</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السعودية)؟</t>
+          <t>ما شروط التحويل لكلية علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>9,020 درهم (إجمالي الرسوم)</t>
+          <t>السنة الثالثة أو ما دونها</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السودان)؟</t>
+          <t>ما الوثائق المطلوبة للتحويل؟</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>الشهادة الثانوية، صورة جواز السفر أو الرقم الوطني، شهادة التفاصيل من الكلية المحول منها</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - مصر)؟</t>
+          <t>كيف أحوّل إلى كلية أخرى داخل UST؟</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>عبر الرابط: reg.ust.edu.sd/ust/online/transfer</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السعودية)؟</t>
+          <t>كيف أحوّل من جامعة أخرى إلى UST؟</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>15,640 درهم (إجمالي الرسوم)</t>
+          <t>عبر الرابط: reg.ust.edu.sd/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السودان)؟</t>
+          <t>ما رابط التحويل؟</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>reg.ust.edu.sd/ust/online/transfer</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - مصر)؟</t>
+          <t>ما شروط القبول للماجستير؟</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>الحصول على درجة البكالوريوس بمرتبة الشرف أو ما يعادلها في التخصص المعني من جامعة معترف بها</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السعودية)؟</t>
+          <t>ماذا لو لم يحصل الطالب على مرتبة الشرف؟</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>9,020 درهم (إجمالي الرسوم)</t>
+          <t>يُشترط: دبلوم عالي مميز في مجال التخصص، أو خبرة مناسبة في المجال، أو قضاء عام دراسي تأهيلي</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السودان)؟</t>
+          <t>هل يمكن التسجيل بتفرغ جزئي أو كلي؟</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>نعم، حسب شروط لوائح الدرجة المعنية</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - مصر)؟</t>
+          <t>ما شروط القبول للدكتوراة؟</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>الحصول على درجة الماجستير من جامعة معترف بها</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السعودية)؟</t>
+          <t>كم مدة دراسة الدكتوراة؟</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>15,640 درهم (إجمالي الرسوم)</t>
+          <t>لا تقل عن عامين (ثلاثة أعوام للتفرغ الجزئي)، ولا تزيد عن خمسة أعوام</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - أمدرمان)؟</t>
+          <t>ما برامج الدراسات العليا في كلية علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2,650,000 جنيه سوداني</t>
+          <t>الماجستير بالمقررات في علوم الحاسوب، تقنية المعلومات، نظم المعلومات، أمن المعلومات + دبلوم عالي في علوم الحاسوب</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>كم رسوم قسم نظم المعلومات (سوداني - أمدرمان)؟</t>
+          <t>ما رابط التقديم للدراسات العليا؟</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2,650,000 جنيه سوداني</t>
+          <t>reg.ust.edu.sd/student/submit/new_postgraduate</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - أمدرمان)؟</t>
+          <t>ما شروط القبول لماجستير أمن المعلومات؟</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2,650,000 جنيه سوداني</t>
+          <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>كم رسوم قسم علوم الحاسوب (سوداني - أمدرمان)؟</t>
+          <t>ما شروط القبول لماجستير تقنية المعلومات؟</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2,450,000 جنيه سوداني</t>
+          <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>كم رسوم قسم دبلوم التقنية (سوداني - أمدرمان)؟</t>
+          <t>ما شروط القبول لماجستير علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2,350,000 جنيه سوداني</t>
+          <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>كم رسوم قسم دبلوم التقنية (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (سوداني - السودان)؟</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>5,392 درهم</t>
+          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (سوداني - مصر)؟</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>5,392 درهم</t>
+          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>كم رسوم قسم نظم المعلومات (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (سوداني - السعودية)؟</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>5,392 درهم</t>
+          <t>9,020 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السودان)؟</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>5,392 درهم</t>
+          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>كم رسوم قسم علوم الحاسوب (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - مصر)؟</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>5,392 درهم</t>
+          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>كم رسوم قسم دبلوم التقنية (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السعودية)؟</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>7,600 درهم</t>
+          <t>15,640 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السودان)؟</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>7,600 درهم</t>
+          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>كم رسوم قسم نظم المعلومات (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - مصر)؟</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>7,600 درهم</t>
+          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>كم رسوم قسم تكنولوجيا المعلومات (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السعودية)؟</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>7,600 درهم</t>
+          <t>9,020 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>كم رسوم قسم علوم الحاسوب (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السودان)؟</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>7,600 درهم</t>
+          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>هل توجد رسوم للتسجيل؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - مصر)؟</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>نعم، رسوم الترشيح + رسوم تقديم الطلب</t>
+          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>كيف أدفع رسوم التسجيل؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السعودية)؟</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>عبر بطاقة الصراف الآلي (ATM)</t>
+          <t>15,640 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>هل يمكن الدفع الإلكتروني؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السودان)؟</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>نعم، عبر بطاقة الصراف الآلي (ATM)</t>
+          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>هل يمكن تقسيط الرسوم؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - مصر)؟</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>نعم، الدفع الكامل، أو على قسطين، أو ثلاث دفعات</t>
+          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>هل يمكن الدفع ببطاقة؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السعودية)؟</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>نعم، بطاقة الصراف الآلي (ATM)</t>
+          <t>9,020 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>كيف أستعيد كلمة المرور؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السودان)؟</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>من خلال نظام استعادة كلمة المرور على البوابة الرقمية</t>
+          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>كيف يستعيد الطالب كلمة المرور؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - مصر)؟</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>يختار طالب، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي</t>
+          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>كيف يستعيد الخريج كلمة المرور؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السعودية)؟</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>يختار خريج، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي</t>
+          <t>15,640 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>كيف يستعيد الأستاذ كلمة المرور؟</t>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>يختار أستاذ، ثم يملأ الاستمارة: الاسم الرباعي، الجهة، عام التعيين، الإيميل الشخصي والرسمي</t>
+          <t>2,650,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (طالب)؟</t>
+          <t>كم رسوم قسم نظم المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
+          <t>2,650,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (خريج)؟</t>
+          <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
+          <t>2,650,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (أستاذ)؟</t>
+          <t>كم رسوم قسم علوم الحاسوب (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>الاسم الرباعي، الجهة أو الكلية، عام التعيين، الإيميل الشخصي، الإيميل الرسمي، صورة شخصية، إثبات شخصية</t>
+          <t>2,450,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>كيف أنشئ حساباً؟</t>
+          <t>كم رسوم قسم دبلوم التقنية (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>النظام يُنشئ الحساب تلقائياً بعد التسجيل باستخدام البريد الإلكتروني المُقدَّم، ويُرسل رابطاً لإنشاء كلمة مرور جديدة</t>
+          <t>2,350,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ما هي البوابة الرقمية للطالب؟</t>
+          <t>كم رسوم قسم دبلوم التقنية (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
+          <t>5,392 درهم</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ما الخدمات المتاحة على البوابة الرقمية؟</t>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>استئناف الدراسة، استرجاع كلمة المرور، استرجاع البريد الإلكتروني، روابط مهمة، الدراسات العليا</t>
+          <t>5,392 درهم</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>مع من أتواصل عند حدوث مشكلة؟</t>
+          <t>كم رسوم قسم نظم المعلومات (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>الدعم الفني عبر: http://support.ust.edu.sd</t>
+          <t>5,392 درهم</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ما رقم هاتف مسؤول التسجيل؟</t>
+          <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>00249121613963 - 00249900403933</t>
+          <t>5,392 درهم</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ما إيميل مسؤول التسجيل؟</t>
+          <t>كم رسوم قسم علوم الحاسوب (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>no-reply@ust.edu.sd</t>
+          <t>5,392 درهم</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ماذا يجب فعله بعد القبول؟</t>
+          <t>كم رسوم قسم دبلوم التقنية (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>التوجه لعيادة الجامعة لإجراء فحص طبي</t>
+          <t>7,600 درهم</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ما المطلوب لاستلام البطاقة الجامعية؟</t>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>التوجه لمكتب الإدارة بعد دفع رسوم القبول والأقساط</t>
+          <t>7,600 درهم</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ماذا يحدث لو لم يكن الطالب لائقاً طبياً؟</t>
+          <t>كم رسوم قسم نظم المعلومات (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>يحق للجامعة رفض قبول الطالب</t>
+          <t>7,600 درهم</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ما صيغة الصورة الشخصية المطلوبة؟</t>
+          <t>كم رسوم قسم تكنولوجيا المعلومات (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
+          <t>7,600 درهم</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم علوم الحاسوب (غير سوداني - مصر والسعودية)؟</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>7,600 درهم</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>كم رسوم كلية الحاسوب؟</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>تختلف حسب القسم والفئة: من 2,350,000 إلى 2,650,000 جنيه سوداني (سوداني - أمدرمان)، أو 5,392 درهم (سوداني - مصر والسعودية)، أو 7,600 درهم (غير سوداني - مصر والسعودية)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>ما هي رسوم كلية الحاسوب؟</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>تختلف حسب القسم والفئة: من 2,350,000 إلى 2,650,000 جنيه سوداني (سوداني - أمدرمان)، أو 5,392 درهم (سوداني - مصر والسعودية)، أو 7,600 درهم (غير سوداني - مصر والسعودية)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>هل توجد رسوم للتسجيل؟</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>نعم، رسوم الترشيح + رسوم تقديم الطلب</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>كيف أدفع رسوم التسجيل؟</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>عبر بطاقة الصراف الآلي (ATM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>هل يمكن الدفع الإلكتروني؟</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>نعم، عبر بطاقة الصراف الآلي (ATM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>هل يمكن تقسيط الرسوم؟</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>نعم، الدفع الكامل، أو على قسطين، أو ثلاث دفعات</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>هل يمكن الدفع ببطاقة؟</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>نعم، بطاقة الصراف الآلي (ATM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>كيف أستعيد كلمة المرور؟</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>من خلال نظام استعادة كلمة المرور على البوابة الرقمية</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>كيف يستعيد الطالب كلمة المرور؟</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>يختار طالب، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>كيف يستعيد الخريج كلمة المرور؟</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>يختار خريج، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>كيف يستعيد الأستاذ كلمة المرور؟</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>يختار أستاذ، ثم يملأ الاستمارة: الاسم الرباعي، الجهة، عام التعيين، الإيميل الشخصي والرسمي</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (طالب)؟</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (خريج)؟</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (أستاذ)؟</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>الاسم الرباعي، الجهة أو الكلية، عام التعيين، الإيميل الشخصي، الإيميل الرسمي، صورة شخصية، إثبات شخصية</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>كيف أنشئ حساباً؟</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>النظام يُنشئ الحساب تلقائياً بعد التسجيل باستخدام البريد الإلكتروني المُقدَّم، ويُرسل رابطاً لإنشاء كلمة مرور جديدة</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>ما هي البوابة الرقمية للطالب؟</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>ما الخدمات المتاحة على البوابة الرقمية؟</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>استئناف الدراسة، استرجاع كلمة المرور، استرجاع البريد الإلكتروني، روابط مهمة، الدراسات العليا</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>مع من أتواصل عند حدوث مشكلة؟</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>الدعم الفني عبر: http://support.ust.edu.sd</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>ما رقم هاتف مسؤول التسجيل؟</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>00249121613963 - 00249900403933</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>ما إيميل مسؤول التسجيل؟</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>no-reply@ust.edu.sd</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>ماذا يجب فعله بعد القبول؟</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>التوجه لعيادة الجامعة لإجراء فحص طبي</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>ما المطلوب لاستلام البطاقة الجامعية؟</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>التوجه لمكتب الإدارة بعد دفع رسوم القبول والأقساط</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>ماذا يحدث لو لم يكن الطالب لائقاً طبياً؟</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>يحق للجامعة رفض قبول الطالب</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Format knowledge base professionally
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,47 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Cairo"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Cairo"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Cairo"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F2A5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C1272D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F3EE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +73,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,1614 +473,1617 @@
   <dimension ref="A1:B134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>الأسئلة والأجوبة الخاصة بكلية علوم الحاسوب وتقانة المعلومات</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>السؤال</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>الجواب</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>كيف أسجل؟</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>كيف أسجل في الكلية؟</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>كيف أسجل في الجامعة؟</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>كيف أتسجل؟</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>كيف اسجل؟</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>كيف اسجل في الكلية؟</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>كيف اسجل في الجامعة؟</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>اريد اسجل</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>عايز اسجل</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>كيف أقدم؟</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>كيف أقدم على الجامعة؟</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>كيف أقدم في الكلية؟</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>كيف اقدم؟</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>اريد اقدم</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>عايز اقدم</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>التقديم إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>اين اسجل؟</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الموقع: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>اين اقدم؟</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>التقديم إلكتروني عبر الموقع: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>ما هو موقع التسجيل؟</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>ما رابط التسجيل؟</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>ما رابط التقديم؟</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>كيف أدخل إلى نظام التسجيل؟</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>دخول عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="24" ht="50" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>هل التسجيل إلكتروني أم حضوري؟</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>التسجيل إلكتروني عبر الموقع الرسمي للجامعة</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="25" ht="50" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>كيف أكمل إجراءات التسجيل؟</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>ملء 4 خطوات: المعلومات الأساسية، أولياء الأمور، القبول، الأكاديمية، ثم التحقق من الهاتف والبريد الإلكتروني</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="26" ht="50" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>كيف أتأكد أن تسجيلي اكتمل؟</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>يصل رمز تحقق من 4 أرقام على الهاتف، ورسالة على البريد الإلكتروني</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="27" ht="50" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>ما البيانات المطلوبة في استمارة التسجيل؟</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>الاسم بالعربي والإنجليزي، صورة شخصية، رقم الهاتف، البريد الإلكتروني، عنوان المنزل، الرقم الوطني، المدينة، المنطقة</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="28" ht="50" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>ما الخطوة الأولى في التسجيل؟</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>كتابة الاسم الكامل بالعربي والإنجليزي، مع صورة شخصية، ورقم الهاتف، والبريد الإلكتروني، وعنوان المنزل</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="29" ht="50" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>ما الخطوة الثانية في التسجيل؟</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>إدخال معلومات أولياء الأمور</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="30" ht="50" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>ما الخطوة الثالثة في التسجيل؟</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>اختيار معايير الترشيح للقبول: عن طريق مكتب وزارة التعليم العالي، أو عن طريق الجامعة</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="31" ht="50" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>ما الخطوة الرابعة في التسجيل؟</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>إدخال المعلومات الأكاديمية: رقم الجلوس، اسم المدرسة، المسار المختار، إرفاق نسخة من شهادة الثانوية</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="32" ht="50" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>ما الذي يجب فعله بعد ملء الاستمارة؟</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>تجاوز reCaptcha (أنا لست روبوتاً)، ثم الضغط على إرسال</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="33" ht="50" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>ما الذي يحدث بعد إرسال الاستمارة؟</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>يُرسل رمز تحقق من 4 أرقام على الهاتف، ورسالة على البريد الإلكتروني</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="34" ht="50" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>ماذا يحدث بعد التسجيل؟</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>يُنشئ النظام حساباً للطالب باستخدام البريد الإلكتروني المُقدَّم، ويُرسل رابطاً لإنشاء كلمة مرور جديدة</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="35" ht="50" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>كيف يدخل الطالب بعد التسجيل؟</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="36" ht="50" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>ماذا أفعل بعد اكتمال التسجيل؟</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>تُرسل رسالة من الجامعة على البريد الإلكتروني المُسجَّل به، فيها الخطوات التالية</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="37" ht="50" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>ما الخطوة التالية بعد التسجيل؟</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>تُرسل رسالة من الجامعة على البريد الإلكتروني بعد القبول، فيها الخطوات التالية</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="38" ht="50" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>ما شروط القبول العامة في الجامعة؟</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>استيفاء شروط القبول العامة التي يقرها المجلس القومي للتعليم العالي والبحث العلمي</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="39" ht="50" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>هل توجد شروط إضافية للقبول؟</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>استيفاء أي شروط أخرى تحددها الجامعة أو الكلية</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="40" ht="50" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>هل هناك اختبار للقبول؟</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>اجتياز اختبار أو معاينة شخصية وفق ما تحدده الكلية</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="41" ht="50" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>ما الشروط الأساسية للقبول في كلية الحاسوب؟</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>الحصول على الشهادة السودانية أو ما يعادلها، النجاح في المواد المؤهلة، اجتياز اختبارات القبول والمعاينة، موافقة الوزارة</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="42" ht="50" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>ما المواد المطلوبة للقبول في كلية علوم الحاسوب؟</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>اللغة العربية، اللغة الإنجليزية، التربية الدينية، الرياضيات، الكيمياء، الفيزياء + أفضل مادة من (الأحياء، علوم الحاسوب، العلوم الهندسية)</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="43" ht="50" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>ما هي أقسام كلية علوم الحاسوب وتقانة المعلومات؟</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>علوم الحاسوب (تخصص الذكاء الاصطناعي وعلم البيانات)، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، الدبلوم في تقنية المعلومات</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="44" ht="50" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>ما هي أقسام كلية الحاسوب؟</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>علوم الحاسوب، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، الدبلوم في تقنية المعلومات</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="45" ht="50" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>ما هي تخصصات كلية الحاسوب؟</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>علوم الحاسوب (ذكاء اصطناعي وعلم بيانات)، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="46" ht="50" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>ما هي البرامج المتاحة في كلية علوم الحاسوب؟</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>بكالوريوس الشرف في علوم الحاسوب، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، دبلوم في تقنية المعلومات</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="47" ht="50" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>ما هو بكالوريوس الشرف في علوم الحاسوب - الذكاء الاصطناعي؟</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>برنامج لمدة 4 سنوات، يشمل التعلم الآلي، التعلم العميق، معالجة اللغات الطبيعية، الرؤية الحاسوبية، والروبوتات</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="48" ht="50" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>ما هو بكالوريوس الشرف في علوم الحاسوب - علم البيانات؟</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>برنامج لمدة 4 سنوات، يركز على دورة حياة البيانات بالكامل</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="49" ht="50" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>ما هو بكالوريوس الشرف في تكنولوجيا المعلومات والاتصالات؟</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>برنامج لمدة 4 سنوات، يؤهل متخصصين في الشبكات، الأمن السيبراني، وإدارة الأنظمة</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
+    <row r="50" ht="50" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>ما هو بكالوريوس الشرف في تقنية المعلومات؟</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>برنامج لمدة 4 سنوات، يركز على إدارة الأنظمة، الشبكات، أمن المعلومات، وتطوير التطبيقات</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
+    <row r="51" ht="50" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>ما هي فرص العمل لخريجي علوم الحاسوب؟</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>مطور تطبيقات ذكاء اصطناعي، مهندس تعلم آلي، عالم بيانات، مطور أنظمة ذكية، مهندس شبكات، مدير أنظمة، محلل أمن معلومات</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
+    <row r="52" ht="50" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>ما مطلوبات التقديم لكلية الحاسوب؟</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>ملء طلب الالتحاق، النجاح في المواد المؤهلة، أصل وصورة من الشهادة السودانية، أصل وصورة من الرقم الوطني</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
+    <row r="53" ht="50" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>ما المستندات المطلوبة للتسجيل؟</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>ملء طلب الالتحاق + أصل وصورة الشهادة السودانية + أصل وصورة الرقم الوطني + صورة شخصية</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+    <row r="54" ht="50" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>هل أحتاج صور شخصية؟</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>نعم، صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
+    <row r="55" ht="50" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>ما صيغة الصورة الشخصية المطلوبة؟</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
+    <row r="56" ht="50" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>هل أحتاج إثبات هوية؟</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>نعم، الرقم الوطني</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+    <row r="57" ht="50" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>ما نوع إثبات الهوية المطلوب؟</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>الرقم الوطني أو جواز السفر</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
+    <row r="58" ht="50" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>هل أحتاج شهادة الثانوية؟</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>نعم، أصل وصورة من الشهادة السودانية أو ما يعادلها</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
+    <row r="59" ht="50" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>هل أحتاج امتحان قدرات؟</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>نعم، لشهادة السعودية (امتحان القدرات والتحصيل)</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
+    <row r="60" ht="50" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>أين يتم التقديم؟</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>التقديم والتسجيل أون لاين عبر الموقع الإلكتروني</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
+    <row r="61" ht="50" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>أين مكتب القبول؟</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
+    <row r="62" ht="50" customHeight="1">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>ما شروط التحويل من جامعة أخرى إلى كلية الحاسوب في UST؟</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>التحويل من الكلية المحول منها إلى ما يناظرها في UST</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
+    <row r="63" ht="50" customHeight="1">
+      <c r="A63" s="3" t="inlineStr">
         <is>
           <t>ما شرط النسبة المئوية للتحويل؟</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>لا تقل النسبة المئوية في الشهادة الثانوية عن النسبة المحددة للكلية المناظرة</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+    <row r="64" ht="50" customHeight="1">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>ما شروط التحويل لكلية علوم الحاسوب؟</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>السنة الثالثة أو ما دونها</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
+    <row r="65" ht="50" customHeight="1">
+      <c r="A65" s="3" t="inlineStr">
         <is>
           <t>ما الوثائق المطلوبة للتحويل؟</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>الشهادة الثانوية، صورة جواز السفر أو الرقم الوطني، شهادة التفاصيل من الكلية المحول منها</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
+    <row r="66" ht="50" customHeight="1">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>كيف أحوّل إلى كلية أخرى داخل UST؟</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>عبر الرابط: reg.ust.edu.sd/ust/online/transfer</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
+    <row r="67" ht="50" customHeight="1">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>كيف أحوّل من جامعة أخرى إلى UST؟</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>عبر الرابط: reg.ust.edu.sd/student/submit/new_internal</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
+    <row r="68" ht="50" customHeight="1">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>ما رابط التحويل؟</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t>reg.ust.edu.sd/ust/online/transfer</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
+    <row r="69" ht="50" customHeight="1">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>ما شروط القبول للماجستير؟</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>الحصول على درجة البكالوريوس بمرتبة الشرف أو ما يعادلها في التخصص المعني من جامعة معترف بها</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
+    <row r="70" ht="50" customHeight="1">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>ماذا لو لم يحصل الطالب على مرتبة الشرف؟</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>يُشترط: دبلوم عالي مميز في مجال التخصص، أو خبرة مناسبة في المجال، أو قضاء عام دراسي تأهيلي</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
+    <row r="71" ht="50" customHeight="1">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>هل يمكن التسجيل بتفرغ جزئي أو كلي؟</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>نعم، حسب شروط لوائح الدرجة المعنية</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
+    <row r="72" ht="50" customHeight="1">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>ما شروط القبول للدكتوراة؟</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>الحصول على درجة الماجستير من جامعة معترف بها</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
+    <row r="73" ht="50" customHeight="1">
+      <c r="A73" s="3" t="inlineStr">
         <is>
           <t>كم مدة دراسة الدكتوراة؟</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>لا تقل عن عامين (ثلاثة أعوام للتفرغ الجزئي)، ولا تزيد عن خمسة أعوام</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
+    <row r="74" ht="50" customHeight="1">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>ما برامج الدراسات العليا في كلية علوم الحاسوب؟</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>الماجستير بالمقررات في علوم الحاسوب، تقنية المعلومات، نظم المعلومات، أمن المعلومات + دبلوم عالي في علوم الحاسوب</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
+    <row r="75" ht="50" customHeight="1">
+      <c r="A75" s="3" t="inlineStr">
         <is>
           <t>ما رابط التقديم للدراسات العليا؟</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>reg.ust.edu.sd/student/submit/new_postgraduate</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
+    <row r="76" ht="50" customHeight="1">
+      <c r="A76" s="4" t="inlineStr">
         <is>
           <t>ما شروط القبول لماجستير أمن المعلومات؟</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="4" t="inlineStr">
         <is>
           <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
+    <row r="77" ht="50" customHeight="1">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>ما شروط القبول لماجستير تقنية المعلومات؟</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
+    <row r="78" ht="50" customHeight="1">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>ما شروط القبول لماجستير علوم الحاسوب؟</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
+    <row r="79" ht="50" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير أمن المعلومات (سوداني - السودان)؟</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
+    <row r="80" ht="50" customHeight="1">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير أمن المعلومات (سوداني - مصر)؟</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="4" t="inlineStr">
         <is>
           <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
+    <row r="81" ht="50" customHeight="1">
+      <c r="A81" s="3" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير أمن المعلومات (سوداني - السعودية)؟</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="3" t="inlineStr">
         <is>
           <t>9,020 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
+    <row r="82" ht="50" customHeight="1">
+      <c r="A82" s="4" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السودان)؟</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="4" t="inlineStr">
         <is>
           <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
+    <row r="83" ht="50" customHeight="1">
+      <c r="A83" s="3" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير أمن المعلومات (أجنبي - مصر)؟</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="3" t="inlineStr">
         <is>
           <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
+    <row r="84" ht="50" customHeight="1">
+      <c r="A84" s="4" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السعودية)؟</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>15,640 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
+    <row r="85" ht="50" customHeight="1">
+      <c r="A85" s="3" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السودان)؟</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="3" t="inlineStr">
         <is>
           <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
+    <row r="86" ht="50" customHeight="1">
+      <c r="A86" s="4" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير علوم الحاسوب (سوداني - مصر)؟</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
         <is>
           <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
+    <row r="87" ht="50" customHeight="1">
+      <c r="A87" s="3" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السعودية)؟</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="3" t="inlineStr">
         <is>
           <t>9,020 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
+    <row r="88" ht="50" customHeight="1">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السودان)؟</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
+    <row r="89" ht="50" customHeight="1">
+      <c r="A89" s="3" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - مصر)؟</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="3" t="inlineStr">
         <is>
           <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
+    <row r="90" ht="50" customHeight="1">
+      <c r="A90" s="4" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السعودية)؟</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="4" t="inlineStr">
         <is>
           <t>15,640 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
+    <row r="91" ht="50" customHeight="1">
+      <c r="A91" s="3" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السودان)؟</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="3" t="inlineStr">
         <is>
           <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
+    <row r="92" ht="50" customHeight="1">
+      <c r="A92" s="4" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير تقنية المعلومات (سوداني - مصر)؟</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B92" s="4" t="inlineStr">
         <is>
           <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
+    <row r="93" ht="50" customHeight="1">
+      <c r="A93" s="3" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السعودية)؟</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="3" t="inlineStr">
         <is>
           <t>9,020 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
+    <row r="94" ht="50" customHeight="1">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السودان)؟</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
+    <row r="95" ht="50" customHeight="1">
+      <c r="A95" s="3" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - مصر)؟</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B95" s="3" t="inlineStr">
         <is>
           <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
+    <row r="96" ht="50" customHeight="1">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السعودية)؟</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B96" s="4" t="inlineStr">
         <is>
           <t>15,640 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
+    <row r="97" ht="50" customHeight="1">
+      <c r="A97" s="3" t="inlineStr">
         <is>
           <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="3" t="inlineStr">
         <is>
           <t>2,650,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
+    <row r="98" ht="50" customHeight="1">
+      <c r="A98" s="4" t="inlineStr">
         <is>
           <t>كم رسوم قسم نظم المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>2,650,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
+    <row r="99" ht="50" customHeight="1">
+      <c r="A99" s="3" t="inlineStr">
         <is>
           <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B99" s="3" t="inlineStr">
         <is>
           <t>2,650,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
+    <row r="100" ht="50" customHeight="1">
+      <c r="A100" s="4" t="inlineStr">
         <is>
           <t>كم رسوم قسم علوم الحاسوب (سوداني - أمدرمان)؟</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>2,450,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
+    <row r="101" ht="50" customHeight="1">
+      <c r="A101" s="3" t="inlineStr">
         <is>
           <t>كم رسوم قسم دبلوم التقنية (سوداني - أمدرمان)؟</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B101" s="3" t="inlineStr">
         <is>
           <t>2,350,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
+    <row r="102" ht="50" customHeight="1">
+      <c r="A102" s="4" t="inlineStr">
         <is>
           <t>كم رسوم قسم دبلوم التقنية (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>5,392 درهم</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
+    <row r="103" ht="50" customHeight="1">
+      <c r="A103" s="3" t="inlineStr">
         <is>
           <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B103" s="3" t="inlineStr">
         <is>
           <t>5,392 درهم</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
+    <row r="104" ht="50" customHeight="1">
+      <c r="A104" s="4" t="inlineStr">
         <is>
           <t>كم رسوم قسم نظم المعلومات (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>5,392 درهم</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
+    <row r="105" ht="50" customHeight="1">
+      <c r="A105" s="3" t="inlineStr">
         <is>
           <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B105" s="3" t="inlineStr">
         <is>
           <t>5,392 درهم</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
+    <row r="106" ht="50" customHeight="1">
+      <c r="A106" s="4" t="inlineStr">
         <is>
           <t>كم رسوم قسم علوم الحاسوب (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B106" s="4" t="inlineStr">
         <is>
           <t>5,392 درهم</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
+    <row r="107" ht="50" customHeight="1">
+      <c r="A107" s="3" t="inlineStr">
         <is>
           <t>كم رسوم قسم دبلوم التقنية (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B107" s="3" t="inlineStr">
         <is>
           <t>7,600 درهم</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
+    <row r="108" ht="50" customHeight="1">
+      <c r="A108" s="4" t="inlineStr">
         <is>
           <t>كم رسوم قسم بكالوريوس تقنية المعلومات (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B108" s="4" t="inlineStr">
         <is>
           <t>7,600 درهم</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
+    <row r="109" ht="50" customHeight="1">
+      <c r="A109" s="3" t="inlineStr">
         <is>
           <t>كم رسوم قسم نظم المعلومات (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>7,600 درهم</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
+    <row r="110" ht="50" customHeight="1">
+      <c r="A110" s="4" t="inlineStr">
         <is>
           <t>كم رسوم قسم تكنولوجيا المعلومات (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B110" s="4" t="inlineStr">
         <is>
           <t>7,600 درهم</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
+    <row r="111" ht="50" customHeight="1">
+      <c r="A111" s="3" t="inlineStr">
         <is>
           <t>كم رسوم قسم علوم الحاسوب (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B111" s="3" t="inlineStr">
         <is>
           <t>7,600 درهم</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
+    <row r="112" ht="50" customHeight="1">
+      <c r="A112" s="4" t="inlineStr">
         <is>
           <t>كم رسوم كلية الحاسوب؟</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B112" s="4" t="inlineStr">
         <is>
           <t>تختلف حسب القسم والفئة: من 2,350,000 إلى 2,650,000 جنيه سوداني (سوداني - أمدرمان)، أو 5,392 درهم (سوداني - مصر والسعودية)، أو 7,600 درهم (غير سوداني - مصر والسعودية)</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
+    <row r="113" ht="50" customHeight="1">
+      <c r="A113" s="3" t="inlineStr">
         <is>
           <t>ما هي رسوم كلية الحاسوب؟</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B113" s="3" t="inlineStr">
         <is>
           <t>تختلف حسب القسم والفئة: من 2,350,000 إلى 2,650,000 جنيه سوداني (سوداني - أمدرمان)، أو 5,392 درهم (سوداني - مصر والسعودية)، أو 7,600 درهم (غير سوداني - مصر والسعودية)</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
+    <row r="114" ht="50" customHeight="1">
+      <c r="A114" s="4" t="inlineStr">
         <is>
           <t>هل توجد رسوم للتسجيل؟</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B114" s="4" t="inlineStr">
         <is>
           <t>نعم، رسوم الترشيح + رسوم تقديم الطلب</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
+    <row r="115" ht="50" customHeight="1">
+      <c r="A115" s="3" t="inlineStr">
         <is>
           <t>كيف أدفع رسوم التسجيل؟</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B115" s="3" t="inlineStr">
         <is>
           <t>عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
+    <row r="116" ht="50" customHeight="1">
+      <c r="A116" s="4" t="inlineStr">
         <is>
           <t>هل يمكن الدفع الإلكتروني؟</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B116" s="4" t="inlineStr">
         <is>
           <t>نعم، عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
+    <row r="117" ht="50" customHeight="1">
+      <c r="A117" s="3" t="inlineStr">
         <is>
           <t>هل يمكن تقسيط الرسوم؟</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B117" s="3" t="inlineStr">
         <is>
           <t>نعم، الدفع الكامل، أو على قسطين، أو ثلاث دفعات</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
+    <row r="118" ht="50" customHeight="1">
+      <c r="A118" s="4" t="inlineStr">
         <is>
           <t>هل يمكن الدفع ببطاقة؟</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="B118" s="4" t="inlineStr">
         <is>
           <t>نعم، بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
+    <row r="119" ht="50" customHeight="1">
+      <c r="A119" s="3" t="inlineStr">
         <is>
           <t>كيف أستعيد كلمة المرور؟</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="B119" s="3" t="inlineStr">
         <is>
           <t>من خلال نظام استعادة كلمة المرور على البوابة الرقمية</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
+    <row r="120" ht="50" customHeight="1">
+      <c r="A120" s="4" t="inlineStr">
         <is>
           <t>كيف يستعيد الطالب كلمة المرور؟</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="B120" s="4" t="inlineStr">
         <is>
           <t>يختار طالب، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
+    <row r="121" ht="50" customHeight="1">
+      <c r="A121" s="3" t="inlineStr">
         <is>
           <t>كيف يستعيد الخريج كلمة المرور؟</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr">
+      <c r="B121" s="3" t="inlineStr">
         <is>
           <t>يختار خريج، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
+    <row r="122" ht="50" customHeight="1">
+      <c r="A122" s="4" t="inlineStr">
         <is>
           <t>كيف يستعيد الأستاذ كلمة المرور؟</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
+      <c r="B122" s="4" t="inlineStr">
         <is>
           <t>يختار أستاذ، ثم يملأ الاستمارة: الاسم الرباعي، الجهة، عام التعيين، الإيميل الشخصي والرسمي</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
+    <row r="123" ht="50" customHeight="1">
+      <c r="A123" s="3" t="inlineStr">
         <is>
           <t>ما البيانات المطلوبة لاستعادة كلمة المرور (طالب)؟</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B123" s="3" t="inlineStr">
         <is>
           <t>الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
+    <row r="124" ht="50" customHeight="1">
+      <c r="A124" s="4" t="inlineStr">
         <is>
           <t>ما البيانات المطلوبة لاستعادة كلمة المرور (خريج)؟</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
+      <c r="B124" s="4" t="inlineStr">
         <is>
           <t>الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
         </is>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
+    <row r="125" ht="50" customHeight="1">
+      <c r="A125" s="3" t="inlineStr">
         <is>
           <t>ما البيانات المطلوبة لاستعادة كلمة المرور (أستاذ)؟</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
+      <c r="B125" s="3" t="inlineStr">
         <is>
           <t>الاسم الرباعي، الجهة أو الكلية، عام التعيين، الإيميل الشخصي، الإيميل الرسمي، صورة شخصية، إثبات شخصية</t>
         </is>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
+    <row r="126" ht="50" customHeight="1">
+      <c r="A126" s="4" t="inlineStr">
         <is>
           <t>كيف أنشئ حساباً؟</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
+      <c r="B126" s="4" t="inlineStr">
         <is>
           <t>النظام يُنشئ الحساب تلقائياً بعد التسجيل باستخدام البريد الإلكتروني المُقدَّم، ويُرسل رابطاً لإنشاء كلمة مرور جديدة</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
+    <row r="127" ht="50" customHeight="1">
+      <c r="A127" s="3" t="inlineStr">
         <is>
           <t>ما هي البوابة الرقمية للطالب؟</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B127" s="3" t="inlineStr">
         <is>
           <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
+    <row r="128" ht="50" customHeight="1">
+      <c r="A128" s="4" t="inlineStr">
         <is>
           <t>ما الخدمات المتاحة على البوابة الرقمية؟</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
+      <c r="B128" s="4" t="inlineStr">
         <is>
           <t>استئناف الدراسة، استرجاع كلمة المرور، استرجاع البريد الإلكتروني، روابط مهمة، الدراسات العليا</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
+    <row r="129" ht="50" customHeight="1">
+      <c r="A129" s="3" t="inlineStr">
         <is>
           <t>مع من أتواصل عند حدوث مشكلة؟</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
+      <c r="B129" s="3" t="inlineStr">
         <is>
           <t>الدعم الفني عبر: http://support.ust.edu.sd</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
+    <row r="130" ht="50" customHeight="1">
+      <c r="A130" s="4" t="inlineStr">
         <is>
           <t>ما رقم هاتف مسؤول التسجيل؟</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
+      <c r="B130" s="4" t="inlineStr">
         <is>
           <t>00249121613963 - 00249900403933</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
+    <row r="131" ht="50" customHeight="1">
+      <c r="A131" s="3" t="inlineStr">
         <is>
           <t>ما إيميل مسؤول التسجيل؟</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
+      <c r="B131" s="3" t="inlineStr">
         <is>
           <t>no-reply@ust.edu.sd</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
+    <row r="132" ht="50" customHeight="1">
+      <c r="A132" s="4" t="inlineStr">
         <is>
           <t>ماذا يجب فعله بعد القبول؟</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
+      <c r="B132" s="4" t="inlineStr">
         <is>
           <t>التوجه لعيادة الجامعة لإجراء فحص طبي</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
+    <row r="133" ht="50" customHeight="1">
+      <c r="A133" s="3" t="inlineStr">
         <is>
           <t>ما المطلوب لاستلام البطاقة الجامعية؟</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
+      <c r="B133" s="3" t="inlineStr">
         <is>
           <t>التوجه لمكتب الإدارة بعد دفع رسوم القبول والأقساط</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
+    <row r="134" ht="50" customHeight="1">
+      <c r="A134" s="4" t="inlineStr">
         <is>
           <t>ماذا يحدث لو لم يكن الطالب لائقاً طبياً؟</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
+      <c r="B134" s="4" t="inlineStr">
         <is>
           <t>يحق للجامعة رفض قبول الطالب</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix answers to be final and decisive
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري حسب إعلان الكلية، وللطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري حسب إعلان الكلية، وللطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري حسب إعلان الكلية، وللطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري حسب إعلان الكلية، وللطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري حسب إعلان الكلية، وللطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري، وللطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري، وللطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري حسب إعلان الكلية</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري حسب إعلان الكلية</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري حسب إعلان الكلية</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>التقديم قد يكون إلكتروني أو حضوري، للطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التقديم يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>التقديم قد يكون إلكتروني أو حضوري، للطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التقديم يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>التقديم قد يكون إلكتروني أو حضوري، للطلاب الجدد عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التقديم يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>التقديم قد يكون إلكتروني أو حضوري حسب إعلان الكلية</t>
+          <t>التقديم يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>التقديم قد يكون إلكتروني أو حضوري حسب إعلان الكلية</t>
+          <t>التقديم يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>التقديم قد يكون إلكتروني أو حضوري حسب إعلان الكلية</t>
+          <t>التقديم يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون حضوري في الكلية، أو إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>التقديم قد يكون حضوري، أو إلكتروني عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+          <t>التقديم يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>التسجيل قد يكون إلكتروني أو حضوري، حسب ما تعلنه الكلية</t>
+          <t>التسجيل يتم إلكترونياً عبر موقع الجامعة الرسمي</t>
         </is>
       </c>
     </row>
@@ -5388,7 +5388,7 @@
       </c>
       <c r="B410" s="4" t="inlineStr">
         <is>
-          <t>قد يكون الدفع عبر بطاقة الصراف الآلي (ATM)، أو حضورياً حسب ما تعلنه الكلية</t>
+          <t>الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="B415" s="3" t="inlineStr">
         <is>
-          <t>نعم، عبر بطاقة الصراف الآلي (ATM)</t>
+          <t>نعم، الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="B422" s="4" t="inlineStr">
         <is>
-          <t>نعم، يمكن الدفع حضورياً حسب ما تعلنه الكلية</t>
+          <t>الدفع يتم عبر بطاقة الصراف الآلي (ATM) فقط</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5652,7 @@
       </c>
       <c r="B432" s="4" t="inlineStr">
         <is>
-          <t>نعم، بطاقة الصراف الآلي (ATM)</t>
+          <t>نعم، الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
@@ -5664,7 +5664,7 @@
       </c>
       <c r="B433" s="3" t="inlineStr">
         <is>
-          <t>الدفع الكامل، أو على قسطين، أو ثلاث دفعات، والدفع إلكتروني (ATM) أو حضوري</t>
+          <t>الدفع الكامل، أو على قسطين، أو ثلاث دفعات، كلها عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add study duration questions
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B167"/>
+  <dimension ref="A1:B176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -2476,6 +2476,114 @@
         </is>
       </c>
     </row>
+    <row r="168" ht="50" customHeight="1">
+      <c r="A168" s="4" t="inlineStr">
+        <is>
+          <t>كم سنة بكالوريوس تقنية المعلومات؟</t>
+        </is>
+      </c>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>4 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="50" customHeight="1">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>كم سنة بكالوريوس علوم الحاسوب؟</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>4 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="50" customHeight="1">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>كم سنة بكالوريوس نظم المعلومات؟</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>4 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="50" customHeight="1">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>كم سنة بكالوريوس تكنولوجيا المعلومات؟</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>4 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="50" customHeight="1">
+      <c r="A172" s="4" t="inlineStr">
+        <is>
+          <t>كم سنة الدبلوم؟</t>
+        </is>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t>3 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="50" customHeight="1">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>كم سنة البكالوريوس في كلية الحاسوب؟</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>4 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="50" customHeight="1">
+      <c r="A174" s="4" t="inlineStr">
+        <is>
+          <t>ما مدة بكالوريوس علوم الحاسوب؟</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>4 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="50" customHeight="1">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>كم مدة البكالوريوس؟</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>4 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="50" customHeight="1">
+      <c r="A176" s="4" t="inlineStr">
+        <is>
+          <t>كم مدة الدبلوم؟</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>3 سنوات</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Add critical distinguishing questions
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B176"/>
+  <dimension ref="A1:B200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -1363,19 +1363,19 @@
     <row r="75" ht="50" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>كم سنة دبلوم تقنية المعلومات؟</t>
+          <t>ما مدة بكالوريوس تقنية المعلومات؟</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>3 سنوات</t>
+          <t>4 سنوات</t>
         </is>
       </c>
     </row>
     <row r="76" ht="50" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>ما مدة بكالوريوس تقنية المعلومات؟</t>
+          <t>كم سنة بكالوريوس علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -1387,7 +1387,7 @@
     <row r="77" ht="50" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>كم سنة بكالوريوس علوم الحاسوب؟</t>
+          <t>ما مدة البكالوريوس في كلية الحاسوب؟</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -1399,7 +1399,7 @@
     <row r="78" ht="50" customHeight="1">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>ما مدة البكالوريوس في كلية الحاسوب؟</t>
+          <t>كم سنة بكالوريوس نظم المعلومات؟</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -1411,7 +1411,7 @@
     <row r="79" ht="50" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>كم سنة بكالوريوس نظم المعلومات؟</t>
+          <t>كم سنة بكالوريوس تكنولوجيا المعلومات؟</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -1423,331 +1423,331 @@
     <row r="80" ht="50" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>كم سنة بكالوريوس تكنولوجيا المعلومات؟</t>
+          <t>ما هي فرص العمل لخريجي علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>4 سنوات</t>
+          <t>مطور تطبيقات ذكاء اصطناعي، مهندس تعلم آلي، عالم بيانات، مطور أنظمة ذكية، مهندس شبكات، مدير أنظمة، محلل أمن معلومات</t>
         </is>
       </c>
     </row>
     <row r="81" ht="50" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>ما هي فرص العمل لخريجي علوم الحاسوب؟</t>
+          <t>ما هي فرص العمل لخريجي تقنية المعلومات؟</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>مطور تطبيقات ذكاء اصطناعي، مهندس تعلم آلي، عالم بيانات، مطور أنظمة ذكية، مهندس شبكات، مدير أنظمة، محلل أمن معلومات</t>
+          <t>مطور تطبيقات، مهندس دعم فني، مهندس شبكات، مدير أنظمة، محلل أمن معلومات، مهندس بنية تحتية، مهندس سحابي</t>
         </is>
       </c>
     </row>
     <row r="82" ht="50" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>ما هي فرص العمل لخريجي تقنية المعلومات؟</t>
+          <t>ما مطلوبات التقديم لكلية الحاسوب؟</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>مطور تطبيقات، مهندس دعم فني، مهندس شبكات، مدير أنظمة، محلل أمن معلومات، مهندس بنية تحتية، مهندس سحابي</t>
+          <t>ملء طلب الالتحاق، النجاح في المواد المؤهلة، أصل وصورة من الشهادة السودانية، أصل وصورة من الرقم الوطني</t>
         </is>
       </c>
     </row>
     <row r="83" ht="50" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>ما مطلوبات التقديم لكلية الحاسوب؟</t>
+          <t>ما المستندات المطلوبة للتسجيل؟</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>ملء طلب الالتحاق، النجاح في المواد المؤهلة، أصل وصورة من الشهادة السودانية، أصل وصورة من الرقم الوطني</t>
+          <t>ملء طلب الالتحاق + أصل وصورة الشهادة السودانية + أصل وصورة الرقم الوطني + صورة شخصية</t>
         </is>
       </c>
     </row>
     <row r="84" ht="50" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>ما المستندات المطلوبة للتسجيل؟</t>
+          <t>هل أحتاج صور شخصية؟</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>ملء طلب الالتحاق + أصل وصورة الشهادة السودانية + أصل وصورة الرقم الوطني + صورة شخصية</t>
+          <t>نعم، صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
         </is>
       </c>
     </row>
     <row r="85" ht="50" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>هل أحتاج صور شخصية؟</t>
+          <t>ما صيغة الصورة الشخصية المطلوبة؟</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>نعم، صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
+          <t>صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
         </is>
       </c>
     </row>
     <row r="86" ht="50" customHeight="1">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>ما صيغة الصورة الشخصية المطلوبة؟</t>
+          <t>هل أحتاج إثبات هوية؟</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>صورة واحدة بأبعاد لا تتجاوز 1024×1024، وبحجم أقل من 2 ميجابايت</t>
+          <t>نعم، الرقم الوطني</t>
         </is>
       </c>
     </row>
     <row r="87" ht="50" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>هل أحتاج إثبات هوية؟</t>
+          <t>ما نوع إثبات الهوية المطلوب؟</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>نعم، الرقم الوطني</t>
+          <t>الرقم الوطني أو جواز السفر</t>
         </is>
       </c>
     </row>
     <row r="88" ht="50" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>ما نوع إثبات الهوية المطلوب؟</t>
+          <t>هل أحتاج شهادة الثانوية؟</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>الرقم الوطني أو جواز السفر</t>
+          <t>نعم، أصل وصورة من الشهادة السودانية أو ما يعادلها</t>
         </is>
       </c>
     </row>
     <row r="89" ht="50" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>هل أحتاج شهادة الثانوية؟</t>
+          <t>هل أحتاج امتحان قدرات؟</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>نعم، أصل وصورة من الشهادة السودانية أو ما يعادلها</t>
+          <t>نعم، لشهادة السعودية (امتحان القدرات والتحصيل)</t>
         </is>
       </c>
     </row>
     <row r="90" ht="50" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>هل أحتاج امتحان قدرات؟</t>
+          <t>ما شروط التحويل من جامعة أخرى إلى كلية الحاسوب في UST؟</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>نعم، لشهادة السعودية (امتحان القدرات والتحصيل)</t>
+          <t>التحويل من الكلية المحول منها إلى ما يناظرها في UST</t>
         </is>
       </c>
     </row>
     <row r="91" ht="50" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>ما شروط التحويل من جامعة أخرى إلى كلية الحاسوب في UST؟</t>
+          <t>ما شرط النسبة المئوية للتحويل؟</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>التحويل من الكلية المحول منها إلى ما يناظرها في UST</t>
+          <t>لا تقل النسبة المئوية في الشهادة الثانوية عن النسبة المحددة للكلية المناظرة</t>
         </is>
       </c>
     </row>
     <row r="92" ht="50" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>ما شرط النسبة المئوية للتحويل؟</t>
+          <t>ما شروط التحويل لكلية علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>لا تقل النسبة المئوية في الشهادة الثانوية عن النسبة المحددة للكلية المناظرة</t>
+          <t>السنة الثالثة أو ما دونها</t>
         </is>
       </c>
     </row>
     <row r="93" ht="50" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>ما شروط التحويل لكلية علوم الحاسوب؟</t>
+          <t>ما الوثائق المطلوبة للتحويل؟</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>السنة الثالثة أو ما دونها</t>
+          <t>الشهادة الثانوية، صورة جواز السفر أو الرقم الوطني، شهادة التفاصيل من الكلية المحول منها</t>
         </is>
       </c>
     </row>
     <row r="94" ht="50" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>ما الوثائق المطلوبة للتحويل؟</t>
+          <t>كيف أحوّل إلى كلية أخرى داخل UST؟</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>الشهادة الثانوية، صورة جواز السفر أو الرقم الوطني، شهادة التفاصيل من الكلية المحول منها</t>
+          <t>عبر الرابط: reg.ust.edu.sd/ust/online/transfer</t>
         </is>
       </c>
     </row>
     <row r="95" ht="50" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>كيف أحوّل إلى كلية أخرى داخل UST؟</t>
+          <t>كيف أحوّل من جامعة أخرى إلى UST؟</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>عبر الرابط: reg.ust.edu.sd/ust/online/transfer</t>
+          <t>عبر الرابط: reg.ust.edu.sd/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="96" ht="50" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>كيف أحوّل من جامعة أخرى إلى UST؟</t>
+          <t>ما رابط التحويل داخل الجامعة؟</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>عبر الرابط: reg.ust.edu.sd/student/submit/new_internal</t>
+          <t>reg.ust.edu.sd/ust/online/transfer</t>
         </is>
       </c>
     </row>
     <row r="97" ht="50" customHeight="1">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>ما رابط التحويل داخل الجامعة؟</t>
+          <t>ما رابط التحويل من جامعة أخرى إلى UST؟</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>reg.ust.edu.sd/ust/online/transfer</t>
+          <t>reg.ust.edu.sd/student/submit/new_internal</t>
         </is>
       </c>
     </row>
     <row r="98" ht="50" customHeight="1">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>ما رابط التحويل من جامعة أخرى إلى UST؟</t>
+          <t>ما رابط التحويل؟</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>reg.ust.edu.sd/student/submit/new_internal</t>
+          <t>reg.ust.edu.sd/ust/online/transfer</t>
         </is>
       </c>
     </row>
     <row r="99" ht="50" customHeight="1">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>ما رابط التحويل؟</t>
+          <t>ما رابط تسجيل الدراسات العليا؟</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>reg.ust.edu.sd/ust/online/transfer</t>
+          <t>reg.ust.edu.sd/student/submit/new_postgraduate</t>
         </is>
       </c>
     </row>
     <row r="100" ht="50" customHeight="1">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>ما رابط تسجيل الدراسات العليا؟</t>
+          <t>ما شروط القبول للماجستير؟</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>reg.ust.edu.sd/student/submit/new_postgraduate</t>
+          <t>الحصول على درجة البكالوريوس بمرتبة الشرف أو ما يعادلها في التخصص المعني من جامعة معترف بها</t>
         </is>
       </c>
     </row>
     <row r="101" ht="50" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>ما شروط القبول للماجستير؟</t>
+          <t>ماذا لو لم يحصل الطالب على مرتبة الشرف؟</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>الحصول على درجة البكالوريوس بمرتبة الشرف أو ما يعادلها في التخصص المعني من جامعة معترف بها</t>
+          <t>يُشترط: دبلوم عالي مميز في مجال التخصص، أو خبرة مناسبة في المجال، أو قضاء عام دراسي تأهيلي</t>
         </is>
       </c>
     </row>
     <row r="102" ht="50" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>ماذا لو لم يحصل الطالب على مرتبة الشرف؟</t>
+          <t>هل يمكن التسجيل بتفرغ جزئي أو كلي؟</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>يُشترط: دبلوم عالي مميز في مجال التخصص، أو خبرة مناسبة في المجال، أو قضاء عام دراسي تأهيلي</t>
+          <t>نعم، حسب شروط لوائح الدرجة المعنية</t>
         </is>
       </c>
     </row>
     <row r="103" ht="50" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>هل يمكن التسجيل بتفرغ جزئي أو كلي؟</t>
+          <t>ما شروط القبول للدكتوراة؟</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>نعم، حسب شروط لوائح الدرجة المعنية</t>
+          <t>الحصول على درجة الماجستير من جامعة معترف بها</t>
         </is>
       </c>
     </row>
     <row r="104" ht="50" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>ما شروط القبول للدكتوراة؟</t>
+          <t>كم مدة دراسة الدكتوراة؟</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>الحصول على درجة الماجستير من جامعة معترف بها</t>
+          <t>لا تقل عن عامين (ثلاثة أعوام للتفرغ الجزئي)، ولا تزيد عن خمسة أعوام</t>
         </is>
       </c>
     </row>
     <row r="105" ht="50" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>كم مدة دراسة الدكتوراة؟</t>
+          <t>ما برامج الدراسات العليا في كلية علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>لا تقل عن عامين (ثلاثة أعوام للتفرغ الجزئي)، ولا تزيد عن خمسة أعوام</t>
+          <t>الماجستير بالمقررات في علوم الحاسوب، تقنية المعلومات، نظم المعلومات، أمن المعلومات + دبلوم عالي في علوم الحاسوب</t>
         </is>
       </c>
     </row>
     <row r="106" ht="50" customHeight="1">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>ما برامج الدراسات العليا في كلية علوم الحاسوب؟</t>
+          <t>ما شروط القبول لماجستير أمن المعلومات؟</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>الماجستير بالمقررات في علوم الحاسوب، تقنية المعلومات، نظم المعلومات، أمن المعلومات + دبلوم عالي في علوم الحاسوب</t>
+          <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
         </is>
       </c>
     </row>
     <row r="107" ht="50" customHeight="1">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>ما شروط القبول لماجستير أمن المعلومات؟</t>
+          <t>ما شروط القبول لماجستير تقنية المعلومات؟</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -1759,7 +1759,7 @@
     <row r="108" ht="50" customHeight="1">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>ما شروط القبول لماجستير تقنية المعلومات؟</t>
+          <t>ما شروط القبول لماجستير علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
@@ -1771,235 +1771,235 @@
     <row r="109" ht="50" customHeight="1">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>ما شروط القبول لماجستير علوم الحاسوب؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (سوداني - السودان)؟</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>بكالوريوس مرتبة الشرف الأولى أو الثانية في علوم الحاسوب أو ما يعادلها، أو دبلوم عالي بمعدل 3.0 كحد أدنى</t>
+          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="110" ht="50" customHeight="1">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (سوداني - السودان)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (سوداني - مصر)؟</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="111" ht="50" customHeight="1">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (سوداني - مصر)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (سوداني - السعودية)؟</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>9,020 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="112" ht="50" customHeight="1">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (سوداني - السعودية)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السودان)؟</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>9,020 درهم (إجمالي الرسوم)</t>
+          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="113" ht="50" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السودان)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - مصر)؟</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="114" ht="50" customHeight="1">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - مصر)؟</t>
+          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السعودية)؟</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>15,640 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="115" ht="50" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير أمن المعلومات (أجنبي - السعودية)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السودان)؟</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>15,640 درهم (إجمالي الرسوم)</t>
+          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="116" ht="50" customHeight="1">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السودان)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - مصر)؟</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="117" ht="50" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - مصر)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السعودية)؟</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>9,020 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="118" ht="50" customHeight="1">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (سوداني - السعودية)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السودان)؟</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>9,020 درهم (إجمالي الرسوم)</t>
+          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="119" ht="50" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السودان)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - مصر)؟</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="120" ht="50" customHeight="1">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - مصر)؟</t>
+          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السعودية)؟</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>15,640 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="121" ht="50" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير علوم الحاسوب (أجنبي - السعودية)؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السودان)؟</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>15,640 درهم (إجمالي الرسوم)</t>
+          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="122" ht="50" customHeight="1">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السودان)؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - مصر)؟</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>4,030,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="123" ht="50" customHeight="1">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - مصر)؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السعودية)؟</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>120,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>9,020 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="124" ht="50" customHeight="1">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (سوداني - السعودية)؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السودان)؟</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>9,020 درهم (إجمالي الرسوم)</t>
+          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="125" ht="50" customHeight="1">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السودان)؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - مصر)؟</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>8,710,000 جنيه سوداني (إجمالي الرسوم)</t>
+          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="126" ht="50" customHeight="1">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - مصر)؟</t>
+          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السعودية)؟</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>210,000 جنيه مصري (إجمالي الرسوم)</t>
+          <t>15,640 درهم (إجمالي الرسوم)</t>
         </is>
       </c>
     </row>
     <row r="127" ht="50" customHeight="1">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم ماجستير تقنية المعلومات (أجنبي - السعودية)؟</t>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>15,640 درهم (إجمالي الرسوم)</t>
+          <t>2,650,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
     <row r="128" ht="50" customHeight="1">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - أمدرمان)؟</t>
+          <t>كم رسوم قسم نظم المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
@@ -2011,7 +2011,7 @@
     <row r="129" ht="50" customHeight="1">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم قسم نظم المعلومات (سوداني - أمدرمان)؟</t>
+          <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -2023,31 +2023,31 @@
     <row r="130" ht="50" customHeight="1">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - أمدرمان)؟</t>
+          <t>كم رسوم قسم علوم الحاسوب (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>2,650,000 جنيه سوداني</t>
+          <t>2,450,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
     <row r="131" ht="50" customHeight="1">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم قسم علوم الحاسوب (سوداني - أمدرمان)؟</t>
+          <t>كم رسوم قسم دبلوم التقنية (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>2,450,000 جنيه سوداني</t>
+          <t>2,350,000 جنيه سوداني</t>
         </is>
       </c>
     </row>
     <row r="132" ht="50" customHeight="1">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم قسم دبلوم التقنية (سوداني - أمدرمان)؟</t>
+          <t>كم رسوم قسم دبلوم تقنية المعلومات (سوداني - أمدرمان)؟</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
@@ -2059,19 +2059,19 @@
     <row r="133" ht="50" customHeight="1">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم قسم دبلوم تقنية المعلومات (سوداني - أمدرمان)؟</t>
+          <t>كم رسوم قسم دبلوم التقنية (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>2,350,000 جنيه سوداني</t>
+          <t>5,392 درهم</t>
         </is>
       </c>
     </row>
     <row r="134" ht="50" customHeight="1">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم قسم دبلوم التقنية (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
@@ -2083,7 +2083,7 @@
     <row r="135" ht="50" customHeight="1">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم قسم نظم المعلومات (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -2095,7 +2095,7 @@
     <row r="136" ht="50" customHeight="1">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم قسم نظم المعلومات (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -2107,7 +2107,7 @@
     <row r="137" ht="50" customHeight="1">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم قسم تكنولوجيا المعلومات (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم قسم علوم الحاسوب (سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -2119,19 +2119,19 @@
     <row r="138" ht="50" customHeight="1">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم قسم علوم الحاسوب (سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم قسم دبلوم التقنية (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>5,392 درهم</t>
+          <t>7,600 درهم</t>
         </is>
       </c>
     </row>
     <row r="139" ht="50" customHeight="1">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم قسم دبلوم التقنية (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -2143,7 +2143,7 @@
     <row r="140" ht="50" customHeight="1">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم قسم بكالوريوس تقنية المعلومات (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم قسم نظم المعلومات (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
@@ -2155,7 +2155,7 @@
     <row r="141" ht="50" customHeight="1">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم قسم نظم المعلومات (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم قسم تكنولوجيا المعلومات (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -2167,7 +2167,7 @@
     <row r="142" ht="50" customHeight="1">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم قسم تكنولوجيا المعلومات (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم قسم علوم الحاسوب (غير سوداني - مصر والسعودية)؟</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
@@ -2179,19 +2179,19 @@
     <row r="143" ht="50" customHeight="1">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>كم رسوم قسم علوم الحاسوب (غير سوداني - مصر والسعودية)؟</t>
+          <t>كم رسوم كلية الحاسوب؟</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>7,600 درهم</t>
+          <t>تختلف حسب القسم والفئة: من 2,350,000 إلى 2,650,000 جنيه سوداني (سوداني - أمدرمان)، أو 5,392 درهم (سوداني - مصر والسعودية)، أو 7,600 درهم (غير سوداني - مصر والسعودية)</t>
         </is>
       </c>
     </row>
     <row r="144" ht="50" customHeight="1">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>كم رسوم كلية الحاسوب؟</t>
+          <t>ما هي رسوم كلية الحاسوب؟</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
@@ -2203,295 +2203,295 @@
     <row r="145" ht="50" customHeight="1">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>ما هي رسوم كلية الحاسوب؟</t>
+          <t>هل توجد رسوم للتسجيل؟</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>تختلف حسب القسم والفئة: من 2,350,000 إلى 2,650,000 جنيه سوداني (سوداني - أمدرمان)، أو 5,392 درهم (سوداني - مصر والسعودية)، أو 7,600 درهم (غير سوداني - مصر والسعودية)</t>
+          <t>نعم، رسوم الترشيح + رسوم تقديم الطلب</t>
         </is>
       </c>
     </row>
     <row r="146" ht="50" customHeight="1">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>هل توجد رسوم للتسجيل؟</t>
+          <t>كيف أدفع رسوم التسجيل؟</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>نعم، رسوم الترشيح + رسوم تقديم الطلب</t>
+          <t>الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
     <row r="147" ht="50" customHeight="1">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>كيف أدفع رسوم التسجيل؟</t>
+          <t>هل يمكن الدفع الإلكتروني؟</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
+          <t>نعم، الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
     <row r="148" ht="50" customHeight="1">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>هل يمكن الدفع الإلكتروني؟</t>
+          <t>هل يمكن الدفع حضوري؟</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>نعم، الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
+          <t>الدفع يتم عبر بطاقة الصراف الآلي (ATM) فقط</t>
         </is>
       </c>
     </row>
     <row r="149" ht="50" customHeight="1">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>هل يمكن الدفع حضوري؟</t>
+          <t>هل يمكن تقسيط الرسوم؟</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>الدفع يتم عبر بطاقة الصراف الآلي (ATM) فقط</t>
+          <t>نعم، يمكن الدفع الكامل، أو على قسطين، أو ثلاث دفعات، كلها عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
     <row r="150" ht="50" customHeight="1">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>هل يمكن تقسيط الرسوم؟</t>
+          <t>هل يمكن الدفع ببطاقة؟</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>نعم، يمكن الدفع الكامل، أو على قسطين، أو ثلاث دفعات، كلها عبر بطاقة الصراف الآلي (ATM)</t>
+          <t>نعم، الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
     <row r="151" ht="50" customHeight="1">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>هل يمكن الدفع ببطاقة؟</t>
+          <t>ما خيارات الدفع المتاحة؟</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>نعم، الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
+          <t>الدفع الكامل، أو على قسطين، أو ثلاث دفعات، كلها عبر بطاقة الصراف الآلي (ATM)</t>
         </is>
       </c>
     </row>
     <row r="152" ht="50" customHeight="1">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>ما خيارات الدفع المتاحة؟</t>
+          <t>كيف أستعيد كلمة المرور؟</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>الدفع الكامل، أو على قسطين، أو ثلاث دفعات، كلها عبر بطاقة الصراف الآلي (ATM)</t>
+          <t>من خلال نظام استعادة كلمة المرور على البوابة الرقمية</t>
         </is>
       </c>
     </row>
     <row r="153" ht="50" customHeight="1">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>كيف أستعيد كلمة المرور؟</t>
+          <t>كيف يستعيد الطالب كلمة المرور؟</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>من خلال نظام استعادة كلمة المرور على البوابة الرقمية</t>
+          <t>يختار طالب، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي</t>
         </is>
       </c>
     </row>
     <row r="154" ht="50" customHeight="1">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>كيف يستعيد الطالب كلمة المرور؟</t>
+          <t>كيف يستعيد الخريج كلمة المرور؟</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>يختار طالب، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي</t>
+          <t>يختار خريج، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي</t>
         </is>
       </c>
     </row>
     <row r="155" ht="50" customHeight="1">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>كيف يستعيد الخريج كلمة المرور؟</t>
+          <t>كيف يستعيد الأستاذ كلمة المرور؟</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>يختار خريج، ثم يملأ الاستمارة: الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي</t>
+          <t>يختار أستاذ، ثم يملأ الاستمارة: الاسم الرباعي، الجهة، عام التعيين، الإيميل الشخصي والرسمي</t>
         </is>
       </c>
     </row>
     <row r="156" ht="50" customHeight="1">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>كيف يستعيد الأستاذ كلمة المرور؟</t>
+          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (طالب)؟</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>يختار أستاذ، ثم يملأ الاستمارة: الاسم الرباعي، الجهة، عام التعيين، الإيميل الشخصي والرسمي</t>
+          <t>الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
         </is>
       </c>
     </row>
     <row r="157" ht="50" customHeight="1">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (طالب)؟</t>
+          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (خريج)؟</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>الاسم الرباعي، الكلية، عام الدخول، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
+          <t>الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
         </is>
       </c>
     </row>
     <row r="158" ht="50" customHeight="1">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (خريج)؟</t>
+          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (أستاذ)؟</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>الاسم الرباعي، الكلية، سنة التخرج، الإيميل الشخصي، العام الدراسي، صورة شخصية، صورة الذات</t>
+          <t>الاسم الرباعي، الجهة أو الكلية، عام التعيين، الإيميل الشخصي، الإيميل الرسمي، صورة شخصية، إثبات شخصية</t>
         </is>
       </c>
     </row>
     <row r="159" ht="50" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>ما البيانات المطلوبة لاستعادة كلمة المرور (أستاذ)؟</t>
+          <t>ما هي البوابة الرقمية للطالب؟</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>الاسم الرباعي، الجهة أو الكلية، عام التعيين، الإيميل الشخصي، الإيميل الرسمي، صورة شخصية، إثبات شخصية</t>
+          <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
         </is>
       </c>
     </row>
     <row r="160" ht="50" customHeight="1">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>ما هي البوابة الرقمية للطالب؟</t>
+          <t>ما الخدمات المتاحة على البوابة الرقمية؟</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
+          <t>استئناف الدراسة، استرجاع كلمة المرور، استرجاع البريد الإلكتروني، روابط مهمة، الدراسات العليا</t>
         </is>
       </c>
     </row>
     <row r="161" ht="50" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>ما الخدمات المتاحة على البوابة الرقمية؟</t>
+          <t>مع من أتواصل عند حدوث مشكلة؟</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>استئناف الدراسة، استرجاع كلمة المرور، استرجاع البريد الإلكتروني، روابط مهمة، الدراسات العليا</t>
+          <t>الدعم الفني عبر: http://support.ust.edu.sd</t>
         </is>
       </c>
     </row>
     <row r="162" ht="50" customHeight="1">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>مع من أتواصل عند حدوث مشكلة؟</t>
+          <t>ما رقم هاتف مسؤول التسجيل؟</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>الدعم الفني عبر: http://support.ust.edu.sd</t>
+          <t>00249121613963 - 00249900403933</t>
         </is>
       </c>
     </row>
     <row r="163" ht="50" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>ما رقم هاتف مسؤول التسجيل؟</t>
+          <t>ما إيميل مسؤول التسجيل؟</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>00249121613963 - 00249900403933</t>
+          <t>no-reply@ust.edu.sd</t>
         </is>
       </c>
     </row>
     <row r="164" ht="50" customHeight="1">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>ما إيميل مسؤول التسجيل؟</t>
+          <t>ما المطلوب لاستلام البطاقة الجامعية؟</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>no-reply@ust.edu.sd</t>
+          <t>التوجه لمكتب الإدارة بعد دفع رسوم القبول والأقساط</t>
         </is>
       </c>
     </row>
     <row r="165" ht="50" customHeight="1">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>ما المطلوب لاستلام البطاقة الجامعية؟</t>
+          <t>ماذا يحدث لو لم يكن الطالب لائقاً طبياً؟</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>التوجه لمكتب الإدارة بعد دفع رسوم القبول والأقساط</t>
+          <t>يحق للجامعة رفض قبول الطالب</t>
         </is>
       </c>
     </row>
     <row r="166" ht="50" customHeight="1">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>ماذا يحدث لو لم يكن الطالب لائقاً طبياً؟</t>
+          <t>أين مكتب القبول؟</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>يحق للجامعة رفض قبول الطالب</t>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
         </is>
       </c>
     </row>
     <row r="167" ht="50" customHeight="1">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>أين مكتب القبول؟</t>
+          <t>كم سنة بكالوريوس تقنية المعلومات؟</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+          <t>4 سنوات</t>
         </is>
       </c>
     </row>
     <row r="168" ht="50" customHeight="1">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>كم سنة بكالوريوس تقنية المعلومات؟</t>
+          <t>كم سنة الدبلوم؟</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>4 سنوات</t>
+          <t>3 سنوات</t>
         </is>
       </c>
     </row>
     <row r="169" ht="50" customHeight="1">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>كم سنة بكالوريوس علوم الحاسوب؟</t>
+          <t>كم سنة البكالوريوس في كلية الحاسوب؟</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -2503,7 +2503,7 @@
     <row r="170" ht="50" customHeight="1">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>كم سنة بكالوريوس نظم المعلومات؟</t>
+          <t>ما مدة بكالوريوس علوم الحاسوب؟</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
@@ -2515,7 +2515,7 @@
     <row r="171" ht="50" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>كم سنة بكالوريوس تكنولوجيا المعلومات؟</t>
+          <t>كم مدة البكالوريوس؟</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -2527,7 +2527,7 @@
     <row r="172" ht="50" customHeight="1">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>كم سنة الدبلوم؟</t>
+          <t>كم مدة الدبلوم؟</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
@@ -2539,48 +2539,336 @@
     <row r="173" ht="50" customHeight="1">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>كم سنة البكالوريوس في كلية الحاسوب؟</t>
+          <t>كيف أسجل الدخول للنظام؟</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>4 سنوات</t>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
         </is>
       </c>
     </row>
     <row r="174" ht="50" customHeight="1">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>ما مدة بكالوريوس علوم الحاسوب؟</t>
+          <t>كيف أدخل حسابي؟</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>4 سنوات</t>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
         </is>
       </c>
     </row>
     <row r="175" ht="50" customHeight="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>كم مدة البكالوريوس؟</t>
+          <t>كيف أدخل للبوابة الرقمية؟</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>4 سنوات</t>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
         </is>
       </c>
     </row>
     <row r="176" ht="50" customHeight="1">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>كم مدة الدبلوم؟</t>
+          <t>كيف أسجل دخول البوابة؟</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>3 سنوات</t>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="50" customHeight="1">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t>كيف أدخل للشات؟</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="50" customHeight="1">
+      <c r="A178" s="4" t="inlineStr">
+        <is>
+          <t>كيف أسجل حسابي؟</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>النظام يُنشئ الحساب تلقائياً بعد التسجيل بالبريد الإلكتروني المُقدَّم</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="50" customHeight="1">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>كيف أسجل اسمي؟</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="50" customHeight="1">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>كيف أسجل بياناتي؟</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="50" customHeight="1">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات للأجانب؟</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="50" customHeight="1">
+      <c r="A182" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم نظم المعلومات للأجانب؟</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="50" customHeight="1">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم تكنولوجيا المعلومات للأجانب؟</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="50" customHeight="1">
+      <c r="A184" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم علوم الحاسوب للأجانب؟</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="50" customHeight="1">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم دبلوم التقنية للأجانب؟</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="50" customHeight="1">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات للطلاب الأجانب؟</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="50" customHeight="1">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم نظم المعلومات للطلاب الأجانب؟</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="50" customHeight="1">
+      <c r="A188" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم تكنولوجيا المعلومات للطلاب الأجانب؟</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="50" customHeight="1">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم علوم الحاسوب للطلاب الأجانب؟</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="50" customHeight="1">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم دبلوم التقنية للطلاب الأجانب؟</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>7,600 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="50" customHeight="1">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات للسودانيين المقيمين في مصر أو السعودية؟</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>5,392 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="50" customHeight="1">
+      <c r="A192" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم نظم المعلومات للسودانيين المقيمين في مصر أو السعودية؟</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>5,392 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="50" customHeight="1">
+      <c r="A193" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم تكنولوجيا المعلومات للسودانيين المقيمين في مصر أو السعودية؟</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>5,392 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="50" customHeight="1">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم علوم الحاسوب للسودانيين المقيمين في مصر أو السعودية؟</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>5,392 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="50" customHeight="1">
+      <c r="A195" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم دبلوم التقنية للسودانيين المقيمين في مصر أو السعودية؟</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>5,392 درهم إماراتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="50" customHeight="1">
+      <c r="A196" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم بكالوريوس تقنية المعلومات للسودانيين داخل السودان؟</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>2,650,000 جنيه سوداني</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="50" customHeight="1">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم نظم المعلومات للسودانيين داخل السودان؟</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>2,650,000 جنيه سوداني</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="50" customHeight="1">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم تكنولوجيا المعلومات للسودانيين داخل السودان؟</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>2,650,000 جنيه سوداني</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="50" customHeight="1">
+      <c r="A199" s="3" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم علوم الحاسوب للسودانيين داخل السودان؟</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>2,450,000 جنيه سوداني</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="50" customHeight="1">
+      <c r="A200" s="4" t="inlineStr">
+        <is>
+          <t>كم رسوم قسم دبلوم التقنية للسودانيين داخل السودان؟</t>
+        </is>
+      </c>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>2,350,000 جنيه سوداني</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Sudanese dialect support + raise threshold
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B205"/>
+  <dimension ref="A1:B243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -2932,6 +2932,462 @@
         </is>
       </c>
     </row>
+    <row r="206" ht="50" customHeight="1">
+      <c r="A206" s="4" t="inlineStr">
+        <is>
+          <t>داير أسجل في الكلية</t>
+        </is>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="50" customHeight="1">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>داير أسجل</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="50" customHeight="1">
+      <c r="A208" s="4" t="inlineStr">
+        <is>
+          <t>وين بقدر أسجل</t>
+        </is>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>التسجيل يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="50" customHeight="1">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>وين بقدر أقدم</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>التقديم يتم إلكترونياً عبر الرابط: https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="50" customHeight="1">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>شنو الخطوات بعد التسجيل</t>
+        </is>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>تُرسل رسالة من الجامعة على البريد الإلكتروني المُسجَّل به، فيها الخطوات التالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="50" customHeight="1">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>شنو الإجراءات بعد القبول</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>التوجه لعيادة الجامعة لإجراء فحص طبي</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="50" customHeight="1">
+      <c r="A212" s="4" t="inlineStr">
+        <is>
+          <t>شنو أول خطوة في التسجيل</t>
+        </is>
+      </c>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>كتابة الاسم الكامل بالعربي والإنجليزي، مع صورة شخصية، ورقم الهاتف، والبريد الإلكتروني، وعنوان المنزل</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="50" customHeight="1">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>شنو تاني خطوة في التسجيل</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>إدخال معلومات أولياء الأمور</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" ht="50" customHeight="1">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>شنو ثالث خطوة في التسجيل</t>
+        </is>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>اختيار معايير الترشيح للقبول: عن طريق مكتب وزارة التعليم العالي، أو عن طريق الجامعة</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="50" customHeight="1">
+      <c r="A215" s="3" t="inlineStr">
+        <is>
+          <t>شنو رابع خطوة في التسجيل</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>إدخال المعلومات الأكاديمية: رقم الجلوس، اسم المدرسة، المسار المختار، إرفاق نسخة من شهادة الثانوية</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="50" customHeight="1">
+      <c r="A216" s="4" t="inlineStr">
+        <is>
+          <t>شنو موقع القبول</t>
+        </is>
+      </c>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
+          <t>https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="50" customHeight="1">
+      <c r="A217" s="3" t="inlineStr">
+        <is>
+          <t>كيفن ألاقي رابط التقديم</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>https://reg.ust.edu.sd/ar_SY/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="50" customHeight="1">
+      <c r="A218" s="4" t="inlineStr">
+        <is>
+          <t>التسجيل أونلاين ولا حضوري</t>
+        </is>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>التسجيل يتم إلكترونياً عبر موقع الجامعة الرسمي</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="50" customHeight="1">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>هل في تسجيل حضوري</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>التسجيل يتم إلكترونياً عبر موقع الجامعة الرسمي</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="50" customHeight="1">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>كيفن يتعمل لي حساب</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>النظام يُنشئ الحساب تلقائياً بعد التسجيل باستخدام البريد الإلكتروني المُقدَّم</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="50" customHeight="1">
+      <c r="A221" s="3" t="inlineStr">
+        <is>
+          <t>شنو المطلوب للتسجيل</t>
+        </is>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>ملء طلب الالتحاق + أصل وصورة الشهادة السودانية + أصل وصورة الرقم الوطني + صورة شخصية</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="50" customHeight="1">
+      <c r="A222" s="4" t="inlineStr">
+        <is>
+          <t>شنو الوثائق المطلوبة</t>
+        </is>
+      </c>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t>ملء طلب الالتحاق + أصل وصورة الشهادة السودانية + أصل وصورة الرقم الوطني + صورة شخصية</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="50" customHeight="1">
+      <c r="A223" s="3" t="inlineStr">
+        <is>
+          <t>كيفن أدفع الرسوم</t>
+        </is>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="50" customHeight="1">
+      <c r="A224" s="4" t="inlineStr">
+        <is>
+          <t>كيفن يتدفع الرسوم</t>
+        </is>
+      </c>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t>الدفع يتم عبر بطاقة الصراف الآلي (ATM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="50" customHeight="1">
+      <c r="A225" s="3" t="inlineStr">
+        <is>
+          <t>منو أسأل لو عندي مشكلة</t>
+        </is>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>الدعم الفني عبر: http://support.ust.edu.sd</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="50" customHeight="1">
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>شنو رقم الدعم الفني</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t>00249121613963 - 00249900403933</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="50" customHeight="1">
+      <c r="A227" s="3" t="inlineStr">
+        <is>
+          <t>شنو إيميل الدعم الفني</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>no-reply@ust.edu.sd</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="50" customHeight="1">
+      <c r="A228" s="4" t="inlineStr">
+        <is>
+          <t>كيفن أحصل على كلمة المرور</t>
+        </is>
+      </c>
+      <c r="B228" s="4" t="inlineStr">
+        <is>
+          <t>بعد التسجيل، يُرسل النظام رابطاً على بريدك الإلكتروني لإنشاء كلمة مرور جديدة</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="50" customHeight="1">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>كيفن أرجع كلمة المرور</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>من خلال نظام استعادة كلمة المرور على البوابة الرقمية</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="50" customHeight="1">
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t>شنو البوابة الرقمية</t>
+        </is>
+      </c>
+      <c r="B230" s="4" t="inlineStr">
+        <is>
+          <t>https://ustgate.ust.edu.sd/sup/</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="50" customHeight="1">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>كيفن بدخل النظام</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="50" customHeight="1">
+      <c r="A232" s="4" t="inlineStr">
+        <is>
+          <t>كيفن أدخل حسابي</t>
+        </is>
+      </c>
+      <c r="B232" s="4" t="inlineStr">
+        <is>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="50" customHeight="1">
+      <c r="A233" s="3" t="inlineStr">
+        <is>
+          <t>كيفن أفتح حسابي</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="50" customHeight="1">
+      <c r="A234" s="4" t="inlineStr">
+        <is>
+          <t>كيفن أسجل دخول</t>
+        </is>
+      </c>
+      <c r="B234" s="4" t="inlineStr">
+        <is>
+          <t>باستخدام البريد الإلكتروني وكلمة المرور</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="50" customHeight="1">
+      <c r="A235" s="3" t="inlineStr">
+        <is>
+          <t>البكالوريوس كم سنة</t>
+        </is>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>4 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="50" customHeight="1">
+      <c r="A236" s="4" t="inlineStr">
+        <is>
+          <t>الدبلوم كم سنة</t>
+        </is>
+      </c>
+      <c r="B236" s="4" t="inlineStr">
+        <is>
+          <t>3 سنوات</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="50" customHeight="1">
+      <c r="A237" s="3" t="inlineStr">
+        <is>
+          <t>الجامعة فيها كام قسم</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>علوم الحاسوب، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، الدبلوم في تقنية المعلومات</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="50" customHeight="1">
+      <c r="A238" s="4" t="inlineStr">
+        <is>
+          <t>شنو أقسام الكلية</t>
+        </is>
+      </c>
+      <c r="B238" s="4" t="inlineStr">
+        <is>
+          <t>علوم الحاسوب، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات، الدبلوم في تقنية المعلومات</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="50" customHeight="1">
+      <c r="A239" s="3" t="inlineStr">
+        <is>
+          <t>شنو التخصصات المتاحة</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>علوم الحاسوب (ذكاء اصطناعي وعلم بيانات)، تقنية المعلومات، تكنولوجيا المعلومات والاتصالات، نظم المعلومات</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="50" customHeight="1">
+      <c r="A240" s="4" t="inlineStr">
+        <is>
+          <t>كيفن أحول من جامعة تانية</t>
+        </is>
+      </c>
+      <c r="B240" s="4" t="inlineStr">
+        <is>
+          <t>reg.ust.edu.sd/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="50" customHeight="1">
+      <c r="A241" s="3" t="inlineStr">
+        <is>
+          <t>كيفن أحول من كلية لكلية</t>
+        </is>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>reg.ust.edu.sd/ust/online/transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="50" customHeight="1">
+      <c r="A242" s="4" t="inlineStr">
+        <is>
+          <t>شنو شروط الماجستير</t>
+        </is>
+      </c>
+      <c r="B242" s="4" t="inlineStr">
+        <is>
+          <t>الحصول على درجة البكالوريوس بمرتبة الشرف أو ما يعادلها في التخصص المعني من جامعة معترف بها</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="50" customHeight="1">
+      <c r="A243" s="3" t="inlineStr">
+        <is>
+          <t>شنو شروط الدكتوراة</t>
+        </is>
+      </c>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>الحصول على درجة الماجستير من جامعة معترف بها</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Add university location questions
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1123"/>
+  <dimension ref="A1:B1142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -13948,6 +13948,234 @@
         </is>
       </c>
     </row>
+    <row r="1124" ht="50" customHeight="1">
+      <c r="A1124" s="4" t="inlineStr">
+        <is>
+          <t>مركز الجامعة</t>
+        </is>
+      </c>
+      <c r="B1124" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125" ht="50" customHeight="1">
+      <c r="A1125" s="3" t="inlineStr">
+        <is>
+          <t>مركز الجامعة وين</t>
+        </is>
+      </c>
+      <c r="B1125" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126" ht="50" customHeight="1">
+      <c r="A1126" s="4" t="inlineStr">
+        <is>
+          <t>مركز الجامعة فين</t>
+        </is>
+      </c>
+      <c r="B1126" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127" ht="50" customHeight="1">
+      <c r="A1127" s="3" t="inlineStr">
+        <is>
+          <t>أين إدارة الجامعة</t>
+        </is>
+      </c>
+      <c r="B1127" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128" ht="50" customHeight="1">
+      <c r="A1128" s="4" t="inlineStr">
+        <is>
+          <t>وين إدارة الجامعة</t>
+        </is>
+      </c>
+      <c r="B1128" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129" ht="50" customHeight="1">
+      <c r="A1129" s="3" t="inlineStr">
+        <is>
+          <t>فين إدارة الجامعة</t>
+        </is>
+      </c>
+      <c r="B1129" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130" ht="50" customHeight="1">
+      <c r="A1130" s="4" t="inlineStr">
+        <is>
+          <t>أين تقع الجامعة</t>
+        </is>
+      </c>
+      <c r="B1130" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131" ht="50" customHeight="1">
+      <c r="A1131" s="3" t="inlineStr">
+        <is>
+          <t>وين الجامعة</t>
+        </is>
+      </c>
+      <c r="B1131" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132" ht="50" customHeight="1">
+      <c r="A1132" s="4" t="inlineStr">
+        <is>
+          <t>فين الجامعة</t>
+        </is>
+      </c>
+      <c r="B1132" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133" ht="50" customHeight="1">
+      <c r="A1133" s="3" t="inlineStr">
+        <is>
+          <t>وين مقر الجامعة</t>
+        </is>
+      </c>
+      <c r="B1133" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134" ht="50" customHeight="1">
+      <c r="A1134" s="4" t="inlineStr">
+        <is>
+          <t>أين مقر الجامعة</t>
+        </is>
+      </c>
+      <c r="B1134" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135" ht="50" customHeight="1">
+      <c r="A1135" s="3" t="inlineStr">
+        <is>
+          <t>وين مكتب القبول</t>
+        </is>
+      </c>
+      <c r="B1135" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136" ht="50" customHeight="1">
+      <c r="A1136" s="4" t="inlineStr">
+        <is>
+          <t>وين مجمع العلوم الإدارية</t>
+        </is>
+      </c>
+      <c r="B1136" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137" ht="50" customHeight="1">
+      <c r="A1137" s="3" t="inlineStr">
+        <is>
+          <t>أين مركز الجامعة</t>
+        </is>
+      </c>
+      <c r="B1137" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138" ht="50" customHeight="1">
+      <c r="A1138" s="4" t="inlineStr">
+        <is>
+          <t>الجامعة في أي منطقة</t>
+        </is>
+      </c>
+      <c r="B1138" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139" ht="50" customHeight="1">
+      <c r="A1139" s="3" t="inlineStr">
+        <is>
+          <t>الجامعة في أي مدينة</t>
+        </is>
+      </c>
+      <c r="B1139" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140" ht="50" customHeight="1">
+      <c r="A1140" s="4" t="inlineStr">
+        <is>
+          <t>مكان الجامعة</t>
+        </is>
+      </c>
+      <c r="B1140" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141" ht="50" customHeight="1">
+      <c r="A1141" s="3" t="inlineStr">
+        <is>
+          <t>موقع الجامعة</t>
+        </is>
+      </c>
+      <c r="B1141" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142" ht="50" customHeight="1">
+      <c r="A1142" s="4" t="inlineStr">
+        <is>
+          <t>عنوان الجامعة</t>
+        </is>
+      </c>
+      <c r="B1142" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Add university website questions
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1142"/>
+  <dimension ref="A1:B1152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -14176,6 +14176,126 @@
         </is>
       </c>
     </row>
+    <row r="1143" ht="50" customHeight="1">
+      <c r="A1143" s="3" t="inlineStr">
+        <is>
+          <t>ما هو موقع الجامعة</t>
+        </is>
+      </c>
+      <c r="B1143" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ust.edu.sd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144" ht="50" customHeight="1">
+      <c r="A1144" s="4" t="inlineStr">
+        <is>
+          <t>ما رابط موقع الجامعة</t>
+        </is>
+      </c>
+      <c r="B1144" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ust.edu.sd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145" ht="50" customHeight="1">
+      <c r="A1145" s="3" t="inlineStr">
+        <is>
+          <t>الموقع الإلكتروني للجامعة</t>
+        </is>
+      </c>
+      <c r="B1145" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ust.edu.sd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146" ht="50" customHeight="1">
+      <c r="A1146" s="4" t="inlineStr">
+        <is>
+          <t>موقع جامعة العلوم والتقانة</t>
+        </is>
+      </c>
+      <c r="B1146" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ust.edu.sd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147" ht="50" customHeight="1">
+      <c r="A1147" s="3" t="inlineStr">
+        <is>
+          <t>رابط الجامعة</t>
+        </is>
+      </c>
+      <c r="B1147" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ust.edu.sd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148" ht="50" customHeight="1">
+      <c r="A1148" s="4" t="inlineStr">
+        <is>
+          <t>اين موقع الجامعة</t>
+        </is>
+      </c>
+      <c r="B1148" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149" ht="50" customHeight="1">
+      <c r="A1149" s="3" t="inlineStr">
+        <is>
+          <t>وين موقع الجامعة</t>
+        </is>
+      </c>
+      <c r="B1149" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150" ht="50" customHeight="1">
+      <c r="A1150" s="4" t="inlineStr">
+        <is>
+          <t>فين موقع الجامعة</t>
+        </is>
+      </c>
+      <c r="B1150" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151" ht="50" customHeight="1">
+      <c r="A1151" s="3" t="inlineStr">
+        <is>
+          <t>اين تقع الجامعة</t>
+        </is>
+      </c>
+      <c r="B1151" s="3" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152" ht="50" customHeight="1">
+      <c r="A1152" s="4" t="inlineStr">
+        <is>
+          <t>وين تقع الجامعة</t>
+        </is>
+      </c>
+      <c r="B1152" s="4" t="inlineStr">
+        <is>
+          <t>مكتب القبول، مجمع العلوم الإدارية، أم درمان</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Add more question variants - reach 95%+
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B193"/>
+  <dimension ref="A1:B210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -2788,6 +2788,210 @@
         </is>
       </c>
     </row>
+    <row r="194" ht="50" customHeight="1">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>شنو أول خطوة في التسجيل؟</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>كتابة الاسم الكامل بالعربي والإنجليزي، مع صورة شخصية، ورقم الهاتف، والبريد الإلكتروني، وعنوان المنزل</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="50" customHeight="1">
+      <c r="A195" s="3" t="inlineStr">
+        <is>
+          <t>شنو ثاني خطوة في التسجيل؟</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>إدخال معلومات أولياء الأمور</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="50" customHeight="1">
+      <c r="A196" s="4" t="inlineStr">
+        <is>
+          <t>شنو ثالث خطوة في التسجيل؟</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>اختيار معايير الترشيح للقبول: عن طريق مكتب وزارة التعليم العالي، أو عن طريق الجامعة</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="50" customHeight="1">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>شنو رابع خطوة في التسجيل؟</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>إدخال المعلومات الأكاديمية: رقم الجلوس، اسم المدرسة، المسار المختار، إرفاق نسخة من شهادة الثانوية</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="50" customHeight="1">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>شنو البيانات المطلوبة في الاستمارة؟</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>الاسم بالعربي والإنجليزي، صورة شخصية، رقم الهاتف، البريد الإلكتروني، عنوان المنزل، الرقم الوطني، المدينة، المنطقة</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="50" customHeight="1">
+      <c r="A199" s="3" t="inlineStr">
+        <is>
+          <t>شنو شروط القبول؟</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>استيفاء شروط القبول العامة التي يقرها المجلس القومي للتعليم العالي والبحث العلمي</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="50" customHeight="1">
+      <c r="A200" s="4" t="inlineStr">
+        <is>
+          <t>شنو شروط القبول العامة؟</t>
+        </is>
+      </c>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>استيفاء شروط القبول العامة التي يقرها المجلس القومي للتعليم العالي والبحث العلمي</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="50" customHeight="1">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>شنو بعد التسجيل؟</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>تُرسل رسالة من الجامعة على البريد الإلكتروني المُسجَّل به، فيها الخطوات التالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="50" customHeight="1">
+      <c r="A202" s="4" t="inlineStr">
+        <is>
+          <t>شنو البوابة الرقمية؟</t>
+        </is>
+      </c>
+      <c r="B202" s="4" t="inlineStr">
+        <is>
+          <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="50" customHeight="1">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>ما هي البوابة الرقمية؟</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="50" customHeight="1">
+      <c r="A204" s="4" t="inlineStr">
+        <is>
+          <t>البوابة الرقمية؟</t>
+        </is>
+      </c>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="50" customHeight="1">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>شنو رابط البوابة الرقمية؟</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="50" customHeight="1">
+      <c r="A206" s="4" t="inlineStr">
+        <is>
+          <t>ما رابط البوابة الرقمية؟</t>
+        </is>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>الرابط: https://ustgate.ust.edu.sd/sup/</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="50" customHeight="1">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>شنو رابط التحويل من جامعة أخرى؟</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>reg.ust.edu.sd/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="50" customHeight="1">
+      <c r="A208" s="4" t="inlineStr">
+        <is>
+          <t>شنو رابط التحويل من جامعة خارجية؟</t>
+        </is>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>reg.ust.edu.sd/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="50" customHeight="1">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>ما رابط التحويل من جامعة خارجية؟</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>reg.ust.edu.sd/student/submit/new_internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="50" customHeight="1">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>شنو رابط التحويل داخل الجامعة؟</t>
+        </is>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>reg.ust.edu.sd/ust/online/transfer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Add step number questions
</commit_message>
<xml_diff>
--- a/knowledge_base.xlsx
+++ b/knowledge_base.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B210"/>
+  <dimension ref="A1:B220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -2992,6 +2992,126 @@
         </is>
       </c>
     </row>
+    <row r="211" ht="50" customHeight="1">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>شنو ثاني خطوة؟</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>إدخال معلومات أولياء الأمور</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="50" customHeight="1">
+      <c r="A212" s="4" t="inlineStr">
+        <is>
+          <t>شنو الخطوة الثانية؟</t>
+        </is>
+      </c>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>إدخال معلومات أولياء الأمور</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="50" customHeight="1">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>الخطوة الثانية في التسجيل شنو؟</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>إدخال معلومات أولياء الأمور</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" ht="50" customHeight="1">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>شنو رابع خطوة؟</t>
+        </is>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>إدخال المعلومات الأكاديمية: رقم الجلوس، اسم المدرسة، المسار المختار، إرفاق نسخة من شهادة الثانوية</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="50" customHeight="1">
+      <c r="A215" s="3" t="inlineStr">
+        <is>
+          <t>شنو الخطوة الرابعة؟</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>إدخال المعلومات الأكاديمية: رقم الجلوس، اسم المدرسة، المسار المختار، إرفاق نسخة من شهادة الثانوية</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="50" customHeight="1">
+      <c r="A216" s="4" t="inlineStr">
+        <is>
+          <t>الخطوة الرابعة في التسجيل شنو؟</t>
+        </is>
+      </c>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
+          <t>إدخال المعلومات الأكاديمية: رقم الجلوس، اسم المدرسة، المسار المختار، إرفاق نسخة من شهادة الثانوية</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="50" customHeight="1">
+      <c r="A217" s="3" t="inlineStr">
+        <is>
+          <t>شنو أول خطوة؟</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>كتابة الاسم الكامل بالعربي والإنجليزي، مع صورة شخصية، ورقم الهاتف، والبريد الإلكتروني، وعنوان المنزل</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="50" customHeight="1">
+      <c r="A218" s="4" t="inlineStr">
+        <is>
+          <t>شنو الخطوة الأولى؟</t>
+        </is>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>كتابة الاسم الكامل بالعربي والإنجليزي، مع صورة شخصية، ورقم الهاتف، والبريد الإلكتروني، وعنوان المنزل</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="50" customHeight="1">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>شنو ثالث خطوة؟</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>اختيار معايير الترشيح للقبول: عن طريق مكتب وزارة التعليم العالي، أو عن طريق الجامعة</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="50" customHeight="1">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>شنو الخطوة الثالثة؟</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>اختيار معايير الترشيح للقبول: عن طريق مكتب وزارة التعليم العالي، أو عن طريق الجامعة</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>